<commit_message>
Fix course template export and Module 20 details
</commit_message>
<xml_diff>
--- a/exports/US History 8-1 - Course Outline.xlsx
+++ b/exports/US History 8-1 - Course Outline.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voyages of Discovery &amp; Commerce and Colonies</t>
+          <t xml:space="preserve">The Voyages of Discovery &amp; Commerce and Colonies</t>
         </is>
       </c>
       <c r="D14" s="16"/>
@@ -661,7 +661,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Voyages of Discovery &amp; Commerce and Colonies</t>
+          <t xml:space="preserve">Overview | The Voyages of Discovery &amp; Commerce and Colonies</t>
         </is>
       </c>
       <c r="D15" s="5"/>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">The French and Indian War &amp; Growing Resentment</t>
+          <t xml:space="preserve">The French and Indian War &amp; Growing Resentment Against Britain</t>
         </is>
       </c>
       <c r="D50" s="16"/>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | The French and Indian War &amp; Growing Resentment</t>
+          <t xml:space="preserve">Overview | The French and Indian War &amp; Growing Resentment Against Britain</t>
         </is>
       </c>
       <c r="D51" s="5"/>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="C188" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROJECT — Dueling Leaders: Burr vs Hamilton  (Project)</t>
+          <t xml:space="preserve">PROJECT - Dueling Leaders: Burr vs Hamilton  (Project)</t>
         </is>
       </c>
       <c r="D188" s="16"/>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="C189" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | PROJECT — Dueling Leaders: Burr vs Hamilton</t>
+          <t xml:space="preserve">Overview | PROJECT - Dueling Leaders: Burr vs Hamilton</t>
         </is>
       </c>
       <c r="D189" s="5"/>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="C289" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+          <t xml:space="preserve">PROJECT - Current Events Connection  (Project)</t>
         </is>
       </c>
       <c r="D289" s="16"/>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="C290" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+          <t xml:space="preserve">Overview | PROJECT - Current Events Connection</t>
         </is>
       </c>
       <c r="D290" s="5"/>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="C296" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midterm Exam  (Exam)</t>
+          <t xml:space="preserve">Study Guide &amp; Final Exam  (Exam)</t>
         </is>
       </c>
       <c r="D296" s="16"/>
@@ -5989,13 +5989,17 @@
       </c>
       <c r="C297" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Midterm Exam</t>
+          <t xml:space="preserve">Overview | Study Guide &amp; Final Exam</t>
         </is>
       </c>
       <c r="D297" s="5"/>
       <c r="E297" s="6"/>
       <c r="F297" s="6"/>
-      <c r="G297" s="6"/>
+      <c r="G297" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semester 1 review and final exam</t>
+        </is>
+      </c>
       <c r="H297" s="2"/>
     </row>
     <row r="298">
@@ -6008,7 +6012,7 @@
       <c r="C298" s="5"/>
       <c r="D298" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Study Guide and Final Exam</t>
         </is>
       </c>
       <c r="E298" s="6"/>
@@ -6020,51 +6024,59 @@
       <c r="A299" s="2"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Page</t>
         </is>
       </c>
       <c r="C299" s="5"/>
-      <c r="D299" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D299" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20.1 | Semester 1 Final Exam Study Guide</t>
         </is>
       </c>
       <c r="E299" s="6"/>
       <c r="F299" s="6"/>
-      <c r="G299" s="6"/>
+      <c r="G299" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Download the study guide, answer the questions in your own words, and study from your answers before the final exam. Download: US History 8-1 Final Exam Study Guide.docx</t>
+        </is>
+      </c>
       <c r="H299" s="2"/>
     </row>
     <row r="300">
       <c r="A300" s="2"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Page</t>
         </is>
       </c>
       <c r="C300" s="5"/>
-      <c r="D300" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D300" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20.2 | Semester 1 Final Exam (Midterm)</t>
         </is>
       </c>
       <c r="E300" s="6"/>
       <c r="F300" s="6"/>
-      <c r="G300" s="6"/>
+      <c r="G300" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Your teacher will tell you when and where to complete the Semester 1 Final Exam. This may also be called the midterm.</t>
+        </is>
+      </c>
       <c r="H300" s="2"/>
     </row>
     <row r="301">
       <c r="A301" s="2"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C301" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Midterm Exam</t>
-        </is>
-      </c>
-      <c r="D301" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C301" s="5"/>
+      <c r="D301" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
+        </is>
+      </c>
       <c r="E301" s="6"/>
       <c r="F301" s="6"/>
       <c r="G301" s="6"/>
@@ -6072,13 +6084,57 @@
     </row>
     <row r="302">
       <c r="A302" s="2"/>
-      <c r="B302" s="2"/>
-      <c r="C302" s="2"/>
-      <c r="D302" s="2"/>
-      <c r="E302" s="2"/>
-      <c r="F302" s="2"/>
-      <c r="G302" s="2"/>
+      <c r="B302" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resource</t>
+        </is>
+      </c>
+      <c r="C302" s="5"/>
+      <c r="D302" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable study guide Word document</t>
+        </is>
+      </c>
+      <c r="E302" s="6"/>
+      <c r="F302" s="6"/>
+      <c r="G302" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">course_planning/content/8-1/module-20-assets/US-History-8-1-Final-Exam-Study-Guide.docx</t>
+        </is>
+      </c>
       <c r="H302" s="2"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="2"/>
+      <c r="B303" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C303" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D303" s="5"/>
+      <c r="E303" s="6"/>
+      <c r="F303" s="6"/>
+      <c r="G303" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module only contains review directions and the downloadable study guide.</t>
+        </is>
+      </c>
+      <c r="H303" s="2"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="2"/>
+      <c r="B304" s="2"/>
+      <c r="C304" s="2"/>
+      <c r="D304" s="2"/>
+      <c r="E304" s="2"/>
+      <c r="F304" s="2"/>
+      <c r="G304" s="2"/>
+      <c r="H304" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">

</xml_diff>

<commit_message>
Add Module 8 DBQ to dashboard
</commit_message>
<xml_diff>
--- a/exports/US History 8-1 - Course Outline.xlsx
+++ b/exports/US History 8-1 - Course Outline.xlsx
@@ -2774,7 +2774,7 @@
       <c r="E126" s="6"/>
       <c r="F126" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HSS 8.2.4, 8.2.6, 8.2.7 | CCSS-ELA RH.1, RH.2, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+          <t xml:space="preserve">HSS 8.2.4, 8.2.6, 8.2.7 | CCSS-ELA RH.1, RH.2, RI.8.8, W.8.1, W.8.4, W.8.9, WHST.1, WHST.4 | ELD Part I A.3, Part I B.6.b</t>
         </is>
       </c>
       <c r="G126" s="6" t="inlineStr">
@@ -2918,22 +2918,18 @@
       <c r="A134" s="2"/>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C134" s="5"/>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">8.3.5 | DBQ: Constitutional Debates</t>
         </is>
       </c>
       <c r="E134" s="6"/>
       <c r="F134" s="6"/>
-      <c r="G134" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 questions</t>
-        </is>
-      </c>
+      <c r="G134" s="6"/>
       <c r="H134" s="2"/>
     </row>
     <row r="135">
@@ -2946,14 +2942,14 @@
       <c r="C135" s="5"/>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: Graded a 'C,' Then He Changed the Constitution</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
       <c r="G135" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 questions</t>
+          <t xml:space="preserve">4 questions</t>
         </is>
       </c>
       <c r="H135" s="2"/>
@@ -2962,143 +2958,147 @@
       <c r="A136" s="2"/>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C136" s="5"/>
-      <c r="D136" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Graded a 'C,' Then He Changed the Constitution</t>
         </is>
       </c>
       <c r="E136" s="6"/>
       <c r="F136" s="6"/>
-      <c r="G136" s="6"/>
+      <c r="G136" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 questions</t>
+        </is>
+      </c>
       <c r="H136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2"/>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C137" s="5"/>
-      <c r="D137" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Ratification &amp; How the Constitution Works</t>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
-      <c r="G137" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G137" s="6"/>
       <c r="H137" s="2"/>
     </row>
     <row r="138">
       <c r="A138" s="2"/>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C138" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Ratification &amp; How the Constitution Works</t>
-        </is>
-      </c>
-      <c r="D138" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C138" s="5"/>
+      <c r="D138" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Ratification &amp; How the Constitution Works</t>
+        </is>
+      </c>
       <c r="E138" s="6"/>
       <c r="F138" s="6"/>
-      <c r="G138" s="6"/>
+      <c r="G138" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H138" s="2"/>
     </row>
     <row r="139">
       <c r="A139" s="2"/>
-      <c r="B139" s="2"/>
-      <c r="C139" s="2"/>
-      <c r="D139" s="2"/>
-      <c r="E139" s="2"/>
-      <c r="F139" s="2"/>
-      <c r="G139" s="2"/>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Ratification &amp; How the Constitution Works</t>
+        </is>
+      </c>
+      <c r="D139" s="5"/>
+      <c r="E139" s="6"/>
+      <c r="F139" s="6"/>
+      <c r="G139" s="6"/>
       <c r="H139" s="2"/>
     </row>
     <row r="140">
       <c r="A140" s="2"/>
-      <c r="B140" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 9</t>
-        </is>
-      </c>
-      <c r="C140" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Federalism &amp; Citizenship</t>
-        </is>
-      </c>
-      <c r="D140" s="16"/>
-      <c r="E140" s="16"/>
-      <c r="F140" s="16"/>
-      <c r="G140" s="17"/>
+      <c r="B140" s="2"/>
+      <c r="C140" s="2"/>
+      <c r="D140" s="2"/>
+      <c r="E140" s="2"/>
+      <c r="F140" s="2"/>
+      <c r="G140" s="2"/>
       <c r="H140" s="2"/>
     </row>
     <row r="141">
       <c r="A141" s="2"/>
-      <c r="B141" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Federalism &amp; Citizenship</t>
-        </is>
-      </c>
-      <c r="D141" s="5"/>
-      <c r="E141" s="6"/>
-      <c r="F141" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.2.3, 8.2.6, 8.3.1, 8.3.6 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
-        </is>
-      </c>
-      <c r="G141" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How does the Constitution divide power between national and state governments, and what rights and responsibilities come with U.S. citizenship?</t>
-        </is>
-      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 9</t>
+        </is>
+      </c>
+      <c r="C141" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Federalism &amp; Citizenship</t>
+        </is>
+      </c>
+      <c r="D141" s="16"/>
+      <c r="E141" s="16"/>
+      <c r="F141" s="16"/>
+      <c r="G141" s="17"/>
       <c r="H141" s="2"/>
     </row>
     <row r="142">
       <c r="A142" s="2"/>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C142" s="5"/>
-      <c r="D142" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Federalism &amp; Citizenship</t>
+        </is>
+      </c>
+      <c r="D142" s="5"/>
       <c r="E142" s="6"/>
-      <c r="F142" s="6"/>
-      <c r="G142" s="6"/>
+      <c r="F142" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.2.3, 8.2.6, 8.3.1, 8.3.6 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+        </is>
+      </c>
+      <c r="G142" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How does the Constitution divide power between national and state governments, and what rights and responsibilities come with U.S. citizenship?</t>
+        </is>
+      </c>
       <c r="H142" s="2"/>
     </row>
     <row r="143">
       <c r="A143" s="2"/>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C143" s="5"/>
-      <c r="D143" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Federalism and Amendments</t>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E143" s="6"/>
@@ -3116,7 +3116,7 @@
       <c r="C144" s="5"/>
       <c r="D144" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Citizens' Rights and Responsibilities</t>
+          <t xml:space="preserve">eText: Federalism and Amendments</t>
         </is>
       </c>
       <c r="E144" s="6"/>
@@ -3128,53 +3128,53 @@
       <c r="A145" s="2"/>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C145" s="5"/>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Federalism and Citizenship</t>
+          <t xml:space="preserve">eText: Citizens' Rights and Responsibilities</t>
         </is>
       </c>
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
-      <c r="G145" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G145" s="6"/>
       <c r="H145" s="2"/>
     </row>
     <row r="146">
       <c r="A146" s="2"/>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C146" s="5"/>
-      <c r="D146" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Federalism and Citizenship</t>
         </is>
       </c>
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
-      <c r="G146" s="6"/>
+      <c r="G146" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H146" s="2"/>
     </row>
     <row r="147">
       <c r="A147" s="2"/>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C147" s="5"/>
-      <c r="D147" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Chart: Methods of Amending the Constitution</t>
+      <c r="D147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E147" s="6"/>
@@ -3192,7 +3192,7 @@
       <c r="C148" s="5"/>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: The First Amendment</t>
+          <t xml:space="preserve">Interactive Chart: Methods of Amending the Constitution</t>
         </is>
       </c>
       <c r="E148" s="6"/>
@@ -3210,7 +3210,7 @@
       <c r="C149" s="5"/>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Voting Responsibly</t>
+          <t xml:space="preserve">Interactive Gallery: The First Amendment</t>
         </is>
       </c>
       <c r="E149" s="6"/>
@@ -3228,7 +3228,7 @@
       <c r="C150" s="5"/>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Civic Responsibility</t>
+          <t xml:space="preserve">Interactive Chart: Voting Responsibly</t>
         </is>
       </c>
       <c r="E150" s="6"/>
@@ -3240,22 +3240,18 @@
       <c r="A151" s="2"/>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C151" s="5"/>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Chart: Civic Responsibility</t>
         </is>
       </c>
       <c r="E151" s="6"/>
       <c r="F151" s="6"/>
-      <c r="G151" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G151" s="6"/>
       <c r="H151" s="2"/>
     </row>
     <row r="152">
@@ -3268,25 +3264,29 @@
       <c r="C152" s="5"/>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: Old Enough to Fight, Too Young to Vote</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
-      <c r="G152" s="6"/>
+      <c r="G152" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H152" s="2"/>
     </row>
     <row r="153">
       <c r="A153" s="2"/>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C153" s="5"/>
-      <c r="D153" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Old Enough to Fight, Too Young to Vote</t>
         </is>
       </c>
       <c r="E153" s="6"/>
@@ -3298,125 +3298,125 @@
       <c r="A154" s="2"/>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C154" s="5"/>
-      <c r="D154" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Federalism &amp; Citizenship</t>
+      <c r="D154" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E154" s="6"/>
       <c r="F154" s="6"/>
-      <c r="G154" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G154" s="6"/>
       <c r="H154" s="2"/>
     </row>
     <row r="155">
       <c r="A155" s="2"/>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Federalism &amp; Citizenship</t>
-        </is>
-      </c>
-      <c r="D155" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C155" s="5"/>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Federalism &amp; Citizenship</t>
+        </is>
+      </c>
       <c r="E155" s="6"/>
       <c r="F155" s="6"/>
-      <c r="G155" s="6"/>
+      <c r="G155" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H155" s="2"/>
     </row>
     <row r="156">
       <c r="A156" s="2"/>
-      <c r="B156" s="2"/>
-      <c r="C156" s="2"/>
-      <c r="D156" s="2"/>
-      <c r="E156" s="2"/>
-      <c r="F156" s="2"/>
-      <c r="G156" s="2"/>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Federalism &amp; Citizenship</t>
+        </is>
+      </c>
+      <c r="D156" s="5"/>
+      <c r="E156" s="6"/>
+      <c r="F156" s="6"/>
+      <c r="G156" s="6"/>
       <c r="H156" s="2"/>
     </row>
     <row r="157">
       <c r="A157" s="2"/>
-      <c r="B157" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 10</t>
-        </is>
-      </c>
-      <c r="C157" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Washington's Presidency &amp; the Two-Party System</t>
-        </is>
-      </c>
-      <c r="D157" s="16"/>
-      <c r="E157" s="16"/>
-      <c r="F157" s="16"/>
-      <c r="G157" s="17"/>
+      <c r="B157" s="2"/>
+      <c r="C157" s="2"/>
+      <c r="D157" s="2"/>
+      <c r="E157" s="2"/>
+      <c r="F157" s="2"/>
+      <c r="G157" s="2"/>
       <c r="H157" s="2"/>
     </row>
     <row r="158">
       <c r="A158" s="2"/>
-      <c r="B158" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C158" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Washington's Presidency &amp; the Two-Party System</t>
-        </is>
-      </c>
-      <c r="D158" s="5"/>
-      <c r="E158" s="6"/>
-      <c r="F158" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
-        </is>
-      </c>
-      <c r="G158" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did Washington shape the presidency, and why did political parties begin to form in the new republic?</t>
-        </is>
-      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 10</t>
+        </is>
+      </c>
+      <c r="C158" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Washington's Presidency &amp; the Two-Party System</t>
+        </is>
+      </c>
+      <c r="D158" s="16"/>
+      <c r="E158" s="16"/>
+      <c r="F158" s="16"/>
+      <c r="G158" s="17"/>
       <c r="H158" s="2"/>
     </row>
     <row r="159">
       <c r="A159" s="2"/>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C159" s="5"/>
-      <c r="D159" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Washington's Presidency &amp; the Two-Party System</t>
+        </is>
+      </c>
+      <c r="D159" s="5"/>
       <c r="E159" s="6"/>
-      <c r="F159" s="6"/>
-      <c r="G159" s="6"/>
+      <c r="F159" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+        </is>
+      </c>
+      <c r="G159" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Washington shape the presidency, and why did political parties begin to form in the new republic?</t>
+        </is>
+      </c>
       <c r="H159" s="2"/>
     </row>
     <row r="160">
       <c r="A160" s="2"/>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C160" s="5"/>
-      <c r="D160" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Washington's Presidency</t>
+      <c r="D160" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E160" s="6"/>
@@ -3434,7 +3434,7 @@
       <c r="C161" s="5"/>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: A Two-Party System Develops</t>
+          <t xml:space="preserve">eText: Washington's Presidency</t>
         </is>
       </c>
       <c r="E161" s="6"/>
@@ -3446,53 +3446,53 @@
       <c r="A162" s="2"/>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C162" s="5"/>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Washington's Presidency and First Political Parties</t>
+          <t xml:space="preserve">eText: A Two-Party System Develops</t>
         </is>
       </c>
       <c r="E162" s="6"/>
       <c r="F162" s="6"/>
-      <c r="G162" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G162" s="6"/>
       <c r="H162" s="2"/>
     </row>
     <row r="163">
       <c r="A163" s="2"/>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C163" s="5"/>
-      <c r="D163" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Washington's Presidency and First Political Parties</t>
         </is>
       </c>
       <c r="E163" s="6"/>
       <c r="F163" s="6"/>
-      <c r="G163" s="6"/>
+      <c r="G163" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H163" s="2"/>
     </row>
     <row r="164">
       <c r="A164" s="2"/>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C164" s="5"/>
-      <c r="D164" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Chart: A Controversial Tax</t>
+      <c r="D164" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E164" s="6"/>
@@ -3510,7 +3510,7 @@
       <c r="C165" s="5"/>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Foreign Affairs Under Washington</t>
+          <t xml:space="preserve">Interactive Chart: A Controversial Tax</t>
         </is>
       </c>
       <c r="E165" s="6"/>
@@ -3528,7 +3528,7 @@
       <c r="C166" s="5"/>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: Early American Leaders</t>
+          <t xml:space="preserve">Interactive Map: Foreign Affairs Under Washington</t>
         </is>
       </c>
       <c r="E166" s="6"/>
@@ -3540,22 +3540,18 @@
       <c r="A167" s="2"/>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C167" s="5"/>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Gallery: Early American Leaders</t>
         </is>
       </c>
       <c r="E167" s="6"/>
       <c r="F167" s="6"/>
-      <c r="G167" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G167" s="6"/>
       <c r="H167" s="2"/>
     </row>
     <row r="168">
@@ -3568,14 +3564,14 @@
       <c r="C168" s="5"/>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: Would You Fight the Government Over Whiskey?</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
       <c r="G168" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">drag-and-drop</t>
+          <t xml:space="preserve">6 questions</t>
         </is>
       </c>
       <c r="H168" s="2"/>
@@ -3584,143 +3580,147 @@
       <c r="A169" s="2"/>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C169" s="5"/>
-      <c r="D169" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Would You Fight the Government Over Whiskey?</t>
         </is>
       </c>
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
-      <c r="G169" s="6"/>
+      <c r="G169" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drag-and-drop</t>
+        </is>
+      </c>
       <c r="H169" s="2"/>
     </row>
     <row r="170">
       <c r="A170" s="2"/>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C170" s="5"/>
-      <c r="D170" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Washington's Presidency &amp; the Two-Party System</t>
+      <c r="D170" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E170" s="6"/>
       <c r="F170" s="6"/>
-      <c r="G170" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G170" s="6"/>
       <c r="H170" s="2"/>
     </row>
     <row r="171">
       <c r="A171" s="2"/>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C171" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Washington's Presidency &amp; the Two-Party System</t>
-        </is>
-      </c>
-      <c r="D171" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C171" s="5"/>
+      <c r="D171" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Washington's Presidency &amp; the Two-Party System</t>
+        </is>
+      </c>
       <c r="E171" s="6"/>
       <c r="F171" s="6"/>
-      <c r="G171" s="6"/>
+      <c r="G171" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H171" s="2"/>
     </row>
     <row r="172">
       <c r="A172" s="2"/>
-      <c r="B172" s="2"/>
-      <c r="C172" s="2"/>
-      <c r="D172" s="2"/>
-      <c r="E172" s="2"/>
-      <c r="F172" s="2"/>
-      <c r="G172" s="2"/>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Washington's Presidency &amp; the Two-Party System</t>
+        </is>
+      </c>
+      <c r="D172" s="5"/>
+      <c r="E172" s="6"/>
+      <c r="F172" s="6"/>
+      <c r="G172" s="6"/>
       <c r="H172" s="2"/>
     </row>
     <row r="173">
       <c r="A173" s="2"/>
-      <c r="B173" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 11</t>
-        </is>
-      </c>
-      <c r="C173" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adams, Jefferson &amp; a Changing Nation</t>
-        </is>
-      </c>
-      <c r="D173" s="16"/>
-      <c r="E173" s="16"/>
-      <c r="F173" s="16"/>
-      <c r="G173" s="17"/>
+      <c r="B173" s="2"/>
+      <c r="C173" s="2"/>
+      <c r="D173" s="2"/>
+      <c r="E173" s="2"/>
+      <c r="F173" s="2"/>
+      <c r="G173" s="2"/>
       <c r="H173" s="2"/>
     </row>
     <row r="174">
       <c r="A174" s="2"/>
-      <c r="B174" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C174" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Adams, Jefferson &amp; a Changing Nation</t>
-        </is>
-      </c>
-      <c r="D174" s="5"/>
-      <c r="E174" s="6"/>
-      <c r="F174" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.4, 8.4.1, 8.5.2, 8.8.2, 8.8.4 | CCSS-ELA RH.1, RH.2, RH.4, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
-        </is>
-      </c>
-      <c r="G174" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did the presidencies of John Adams and Thomas Jefferson test the young nation's political ideas, rights, and expansion?</t>
-        </is>
-      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 11</t>
+        </is>
+      </c>
+      <c r="C174" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adams, Jefferson &amp; a Changing Nation</t>
+        </is>
+      </c>
+      <c r="D174" s="16"/>
+      <c r="E174" s="16"/>
+      <c r="F174" s="16"/>
+      <c r="G174" s="17"/>
       <c r="H174" s="2"/>
     </row>
     <row r="175">
       <c r="A175" s="2"/>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C175" s="5"/>
-      <c r="D175" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Adams, Jefferson &amp; a Changing Nation</t>
+        </is>
+      </c>
+      <c r="D175" s="5"/>
       <c r="E175" s="6"/>
-      <c r="F175" s="6"/>
-      <c r="G175" s="6"/>
+      <c r="F175" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.4, 8.4.1, 8.5.2, 8.8.2, 8.8.4 | CCSS-ELA RH.1, RH.2, RH.4, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+        </is>
+      </c>
+      <c r="G175" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did the presidencies of John Adams and Thomas Jefferson test the young nation's political ideas, rights, and expansion?</t>
+        </is>
+      </c>
       <c r="H175" s="2"/>
     </row>
     <row r="176">
       <c r="A176" s="2"/>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C176" s="5"/>
-      <c r="D176" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Presidents Adams and Jefferson</t>
+      <c r="D176" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E176" s="6"/>
@@ -3738,7 +3738,7 @@
       <c r="C177" s="5"/>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: A Changing Nation</t>
+          <t xml:space="preserve">eText: Presidents Adams and Jefferson</t>
         </is>
       </c>
       <c r="E177" s="6"/>
@@ -3750,53 +3750,53 @@
       <c r="A178" s="2"/>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C178" s="5"/>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Adams, Jefferson, and Expansion</t>
+          <t xml:space="preserve">eText: A Changing Nation</t>
         </is>
       </c>
       <c r="E178" s="6"/>
       <c r="F178" s="6"/>
-      <c r="G178" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G178" s="6"/>
       <c r="H178" s="2"/>
     </row>
     <row r="179">
       <c r="A179" s="2"/>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C179" s="5"/>
-      <c r="D179" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D179" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Adams, Jefferson, and Expansion</t>
         </is>
       </c>
       <c r="E179" s="6"/>
       <c r="F179" s="6"/>
-      <c r="G179" s="6"/>
+      <c r="G179" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H179" s="2"/>
     </row>
     <row r="180">
       <c r="A180" s="2"/>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C180" s="5"/>
-      <c r="D180" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Chart: Hamilton, Adams, or Jefferson?</t>
+      <c r="D180" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E180" s="6"/>
@@ -3814,7 +3814,7 @@
       <c r="C181" s="5"/>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Expansion and Exploration</t>
+          <t xml:space="preserve">Interactive Chart: Hamilton, Adams, or Jefferson?</t>
         </is>
       </c>
       <c r="E181" s="6"/>
@@ -3826,22 +3826,18 @@
       <c r="A182" s="2"/>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C182" s="5"/>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Map: Expansion and Exploration</t>
         </is>
       </c>
       <c r="E182" s="6"/>
       <c r="F182" s="6"/>
-      <c r="G182" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G182" s="6"/>
       <c r="H182" s="2"/>
     </row>
     <row r="183">
@@ -3854,14 +3850,14 @@
       <c r="C183" s="5"/>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: Jefferson's Monster Map</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
       <c r="G183" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 questions</t>
+          <t xml:space="preserve">6 questions</t>
         </is>
       </c>
       <c r="H183" s="2"/>
@@ -3870,170 +3866,174 @@
       <c r="A184" s="2"/>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C184" s="5"/>
-      <c r="D184" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Jefferson's Monster Map</t>
         </is>
       </c>
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
-      <c r="G184" s="6"/>
+      <c r="G184" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 questions</t>
+        </is>
+      </c>
       <c r="H184" s="2"/>
     </row>
     <row r="185">
       <c r="A185" s="2"/>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C185" s="5"/>
-      <c r="D185" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Adams, Jefferson &amp; a Changing Nation</t>
+      <c r="D185" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
-      <c r="G185" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G185" s="6"/>
       <c r="H185" s="2"/>
     </row>
     <row r="186">
       <c r="A186" s="2"/>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C186" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Adams, Jefferson &amp; a Changing Nation</t>
-        </is>
-      </c>
-      <c r="D186" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C186" s="5"/>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Adams, Jefferson &amp; a Changing Nation</t>
+        </is>
+      </c>
       <c r="E186" s="6"/>
       <c r="F186" s="6"/>
-      <c r="G186" s="6"/>
+      <c r="G186" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H186" s="2"/>
     </row>
     <row r="187">
       <c r="A187" s="2"/>
-      <c r="B187" s="2"/>
-      <c r="C187" s="2"/>
-      <c r="D187" s="2"/>
-      <c r="E187" s="2"/>
-      <c r="F187" s="2"/>
-      <c r="G187" s="2"/>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C187" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Adams, Jefferson &amp; a Changing Nation</t>
+        </is>
+      </c>
+      <c r="D187" s="5"/>
+      <c r="E187" s="6"/>
+      <c r="F187" s="6"/>
+      <c r="G187" s="6"/>
       <c r="H187" s="2"/>
     </row>
     <row r="188">
       <c r="A188" s="2"/>
-      <c r="B188" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 12</t>
-        </is>
-      </c>
-      <c r="C188" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT - Dueling Leaders: Burr vs Hamilton  (Project)</t>
-        </is>
-      </c>
-      <c r="D188" s="16"/>
-      <c r="E188" s="16"/>
-      <c r="F188" s="16"/>
-      <c r="G188" s="17"/>
+      <c r="B188" s="2"/>
+      <c r="C188" s="2"/>
+      <c r="D188" s="2"/>
+      <c r="E188" s="2"/>
+      <c r="F188" s="2"/>
+      <c r="G188" s="2"/>
       <c r="H188" s="2"/>
     </row>
     <row r="189">
       <c r="A189" s="2"/>
-      <c r="B189" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C189" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT - Dueling Leaders: Burr vs Hamilton</t>
-        </is>
-      </c>
-      <c r="D189" s="5"/>
-      <c r="E189" s="6"/>
-      <c r="F189" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.9, WHST.1, WHST.4 | ELD Part I A.3, Part I B.6, Part I C.10, Part I C.11</t>
-        </is>
-      </c>
-      <c r="G189" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Should Aaron Burr have been found criminally responsible for Alexander Hamilton's death?</t>
-        </is>
-      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 12</t>
+        </is>
+      </c>
+      <c r="C189" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Dueling Leaders: Burr vs Hamilton  (Project)</t>
+        </is>
+      </c>
+      <c r="D189" s="16"/>
+      <c r="E189" s="16"/>
+      <c r="F189" s="16"/>
+      <c r="G189" s="17"/>
       <c r="H189" s="2"/>
     </row>
     <row r="190">
       <c r="A190" s="2"/>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C190" s="5"/>
-      <c r="D190" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C190" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT - Dueling Leaders: Burr vs Hamilton</t>
+        </is>
+      </c>
+      <c r="D190" s="5"/>
       <c r="E190" s="6"/>
-      <c r="F190" s="6"/>
-      <c r="G190" s="6"/>
+      <c r="F190" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.9, WHST.1, WHST.4 | ELD Part I A.3, Part I B.6, Part I C.10, Part I C.11</t>
+        </is>
+      </c>
+      <c r="G190" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Should Aaron Burr have been found criminally responsible for Alexander Hamilton's death?</t>
+        </is>
+      </c>
       <c r="H190" s="2"/>
     </row>
     <row r="191">
       <c r="A191" s="2"/>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C191" s="5"/>
-      <c r="D191" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Video: Hamilton and Burr: The Duel That Became a Case File</t>
+      <c r="D191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
-      <c r="G191" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 check questions</t>
-        </is>
-      </c>
+      <c r="G191" s="6"/>
       <c r="H191" s="2"/>
     </row>
     <row r="192">
       <c r="A192" s="2"/>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C192" s="5"/>
-      <c r="D192" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D192" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Hamilton and Burr: The Duel That Became a Case File</t>
         </is>
       </c>
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
-      <c r="G192" s="6"/>
+      <c r="G192" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 check questions</t>
+        </is>
+      </c>
       <c r="H192" s="2"/>
     </row>
     <row r="193">
@@ -4046,7 +4046,7 @@
       <c r="C193" s="5"/>
       <c r="D193" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E193" s="6"/>
@@ -4058,15 +4058,15 @@
       <c r="A194" s="2"/>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C194" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Dueling Leaders: Burr vs Hamilton</t>
-        </is>
-      </c>
-      <c r="D194" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C194" s="5"/>
+      <c r="D194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
@@ -4074,87 +4074,87 @@
     </row>
     <row r="195">
       <c r="A195" s="2"/>
-      <c r="B195" s="2"/>
-      <c r="C195" s="2"/>
-      <c r="D195" s="2"/>
-      <c r="E195" s="2"/>
-      <c r="F195" s="2"/>
-      <c r="G195" s="2"/>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C195" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Dueling Leaders: Burr vs Hamilton</t>
+        </is>
+      </c>
+      <c r="D195" s="5"/>
+      <c r="E195" s="6"/>
+      <c r="F195" s="6"/>
+      <c r="G195" s="6"/>
       <c r="H195" s="2"/>
     </row>
     <row r="196">
       <c r="A196" s="2"/>
-      <c r="B196" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 13</t>
-        </is>
-      </c>
-      <c r="C196" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Madison &amp; the War of 1812</t>
-        </is>
-      </c>
-      <c r="D196" s="16"/>
-      <c r="E196" s="16"/>
-      <c r="F196" s="16"/>
-      <c r="G196" s="17"/>
+      <c r="B196" s="2"/>
+      <c r="C196" s="2"/>
+      <c r="D196" s="2"/>
+      <c r="E196" s="2"/>
+      <c r="F196" s="2"/>
+      <c r="G196" s="2"/>
       <c r="H196" s="2"/>
     </row>
     <row r="197">
       <c r="A197" s="2"/>
-      <c r="B197" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C197" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Madison &amp; the War of 1812</t>
-        </is>
-      </c>
-      <c r="D197" s="5"/>
-      <c r="E197" s="6"/>
-      <c r="F197" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.5.1, 8.5.2, 8.5.3, 8.12.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G197" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Why did the United States go to war with Britain in 1812, and how did the war change Americans' sense of national identity?</t>
-        </is>
-      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 13</t>
+        </is>
+      </c>
+      <c r="C197" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Madison &amp; the War of 1812</t>
+        </is>
+      </c>
+      <c r="D197" s="16"/>
+      <c r="E197" s="16"/>
+      <c r="F197" s="16"/>
+      <c r="G197" s="17"/>
       <c r="H197" s="2"/>
     </row>
     <row r="198">
       <c r="A198" s="2"/>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C198" s="5"/>
-      <c r="D198" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C198" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Madison &amp; the War of 1812</t>
+        </is>
+      </c>
+      <c r="D198" s="5"/>
       <c r="E198" s="6"/>
-      <c r="F198" s="6"/>
-      <c r="G198" s="6"/>
+      <c r="F198" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.5.1, 8.5.2, 8.5.3, 8.12.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G198" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why did the United States go to war with Britain in 1812, and how did the war change Americans' sense of national identity?</t>
+        </is>
+      </c>
       <c r="H198" s="2"/>
     </row>
     <row r="199">
       <c r="A199" s="2"/>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C199" s="5"/>
-      <c r="D199" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Madison and the War of 1812</t>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E199" s="6"/>
@@ -4166,53 +4166,53 @@
       <c r="A200" s="2"/>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C200" s="5"/>
       <c r="D200" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Causes and Symbols of the War of 1812</t>
+          <t xml:space="preserve">eText: Madison and the War of 1812</t>
         </is>
       </c>
       <c r="E200" s="6"/>
       <c r="F200" s="6"/>
-      <c r="G200" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G200" s="6"/>
       <c r="H200" s="2"/>
     </row>
     <row r="201">
       <c r="A201" s="2"/>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C201" s="5"/>
-      <c r="D201" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D201" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Causes and Symbols of the War of 1812</t>
         </is>
       </c>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
-      <c r="G201" s="6"/>
+      <c r="G201" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H201" s="2"/>
     </row>
     <row r="202">
       <c r="A202" s="2"/>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C202" s="5"/>
-      <c r="D202" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Map: Indian Lands Lost by 1810</t>
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E202" s="6"/>
@@ -4230,7 +4230,7 @@
       <c r="C203" s="5"/>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: The War of 1812</t>
+          <t xml:space="preserve">Interactive Map: Indian Lands Lost by 1810</t>
         </is>
       </c>
       <c r="E203" s="6"/>
@@ -4242,22 +4242,18 @@
       <c r="A204" s="2"/>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C204" s="5"/>
       <c r="D204" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Map: The War of 1812</t>
         </is>
       </c>
       <c r="E204" s="6"/>
       <c r="F204" s="6"/>
-      <c r="G204" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G204" s="6"/>
       <c r="H204" s="2"/>
     </row>
     <row r="205">
@@ -4270,25 +4266,29 @@
       <c r="C205" s="5"/>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Battle After the Treaty</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
-      <c r="G205" s="6"/>
+      <c r="G205" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H205" s="2"/>
     </row>
     <row r="206">
       <c r="A206" s="2"/>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C206" s="5"/>
-      <c r="D206" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Battle After the Treaty</t>
         </is>
       </c>
       <c r="E206" s="6"/>
@@ -4300,125 +4300,125 @@
       <c r="A207" s="2"/>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C207" s="5"/>
-      <c r="D207" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Madison &amp; the War of 1812</t>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E207" s="6"/>
       <c r="F207" s="6"/>
-      <c r="G207" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G207" s="6"/>
       <c r="H207" s="2"/>
     </row>
     <row r="208">
       <c r="A208" s="2"/>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C208" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Madison &amp; the War of 1812</t>
-        </is>
-      </c>
-      <c r="D208" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C208" s="5"/>
+      <c r="D208" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Madison &amp; the War of 1812</t>
+        </is>
+      </c>
       <c r="E208" s="6"/>
       <c r="F208" s="6"/>
-      <c r="G208" s="6"/>
+      <c r="G208" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H208" s="2"/>
     </row>
     <row r="209">
       <c r="A209" s="2"/>
-      <c r="B209" s="2"/>
-      <c r="C209" s="2"/>
-      <c r="D209" s="2"/>
-      <c r="E209" s="2"/>
-      <c r="F209" s="2"/>
-      <c r="G209" s="2"/>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C209" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Madison &amp; the War of 1812</t>
+        </is>
+      </c>
+      <c r="D209" s="5"/>
+      <c r="E209" s="6"/>
+      <c r="F209" s="6"/>
+      <c r="G209" s="6"/>
       <c r="H209" s="2"/>
     </row>
     <row r="210">
       <c r="A210" s="2"/>
-      <c r="B210" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 14</t>
-        </is>
-      </c>
-      <c r="C210" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Monroe's Presidency and Everyday Life</t>
-        </is>
-      </c>
-      <c r="D210" s="16"/>
-      <c r="E210" s="16"/>
-      <c r="F210" s="16"/>
-      <c r="G210" s="17"/>
+      <c r="B210" s="2"/>
+      <c r="C210" s="2"/>
+      <c r="D210" s="2"/>
+      <c r="E210" s="2"/>
+      <c r="F210" s="2"/>
+      <c r="G210" s="2"/>
       <c r="H210" s="2"/>
     </row>
     <row r="211">
       <c r="A211" s="2"/>
-      <c r="B211" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C211" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Monroe's Presidency and Everyday Life</t>
-        </is>
-      </c>
-      <c r="D211" s="5"/>
-      <c r="E211" s="6"/>
-      <c r="F211" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.3, 8.4.1, 8.4.3, 8.4.4, 8.5.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G211" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did the United States grow stronger, more connected, and more divided during Monroe's presidency and the early 1800s?</t>
-        </is>
-      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 14</t>
+        </is>
+      </c>
+      <c r="C211" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
+      <c r="D211" s="16"/>
+      <c r="E211" s="16"/>
+      <c r="F211" s="16"/>
+      <c r="G211" s="17"/>
       <c r="H211" s="2"/>
     </row>
     <row r="212">
       <c r="A212" s="2"/>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C212" s="5"/>
-      <c r="D212" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C212" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
+      <c r="D212" s="5"/>
       <c r="E212" s="6"/>
-      <c r="F212" s="6"/>
-      <c r="G212" s="6"/>
+      <c r="F212" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.3, 8.4.1, 8.4.3, 8.4.4, 8.5.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G212" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did the United States grow stronger, more connected, and more divided during Monroe's presidency and the early 1800s?</t>
+        </is>
+      </c>
       <c r="H212" s="2"/>
     </row>
     <row r="213">
       <c r="A213" s="2"/>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C213" s="5"/>
-      <c r="D213" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Monroe's Presidency and Everyday Life</t>
+      <c r="D213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E213" s="6"/>
@@ -4430,53 +4430,53 @@
       <c r="A214" s="2"/>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C214" s="5"/>
       <c r="D214" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: The Erie Canal and National Growth</t>
+          <t xml:space="preserve">eText: Monroe's Presidency and Everyday Life</t>
         </is>
       </c>
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
-      <c r="G214" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G214" s="6"/>
       <c r="H214" s="2"/>
     </row>
     <row r="215">
       <c r="A215" s="2"/>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C215" s="5"/>
-      <c r="D215" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: The Erie Canal and National Growth</t>
         </is>
       </c>
       <c r="E215" s="6"/>
       <c r="F215" s="6"/>
-      <c r="G215" s="6"/>
+      <c r="G215" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H215" s="2"/>
     </row>
     <row r="216">
       <c r="A216" s="2"/>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C216" s="5"/>
-      <c r="D216" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Chart: The Beginnings of Sectionalism</t>
+      <c r="D216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E216" s="6"/>
@@ -4494,7 +4494,7 @@
       <c r="C217" s="5"/>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: The Expansion of Federal Power</t>
+          <t xml:space="preserve">Interactive Chart: The Beginnings of Sectionalism</t>
         </is>
       </c>
       <c r="E217" s="6"/>
@@ -4506,22 +4506,18 @@
       <c r="A218" s="2"/>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C218" s="5"/>
       <c r="D218" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Gallery: The Expansion of Federal Power</t>
         </is>
       </c>
       <c r="E218" s="6"/>
       <c r="F218" s="6"/>
-      <c r="G218" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G218" s="6"/>
       <c r="H218" s="2"/>
     </row>
     <row r="219">
@@ -4534,25 +4530,29 @@
       <c r="C219" s="5"/>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Canal Wedding That Changed America</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E219" s="6"/>
       <c r="F219" s="6"/>
-      <c r="G219" s="6"/>
+      <c r="G219" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H219" s="2"/>
     </row>
     <row r="220">
       <c r="A220" s="2"/>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C220" s="5"/>
-      <c r="D220" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D220" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Canal Wedding That Changed America</t>
         </is>
       </c>
       <c r="E220" s="6"/>
@@ -4564,125 +4564,125 @@
       <c r="A221" s="2"/>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C221" s="5"/>
-      <c r="D221" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Monroe's Presidency and Everyday Life</t>
+      <c r="D221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E221" s="6"/>
       <c r="F221" s="6"/>
-      <c r="G221" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G221" s="6"/>
       <c r="H221" s="2"/>
     </row>
     <row r="222">
       <c r="A222" s="2"/>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C222" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Monroe's Presidency and Everyday Life</t>
-        </is>
-      </c>
-      <c r="D222" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C222" s="5"/>
+      <c r="D222" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
       <c r="E222" s="6"/>
       <c r="F222" s="6"/>
-      <c r="G222" s="6"/>
+      <c r="G222" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H222" s="2"/>
     </row>
     <row r="223">
       <c r="A223" s="2"/>
-      <c r="B223" s="2"/>
-      <c r="C223" s="2"/>
-      <c r="D223" s="2"/>
-      <c r="E223" s="2"/>
-      <c r="F223" s="2"/>
-      <c r="G223" s="2"/>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C223" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
+      <c r="D223" s="5"/>
+      <c r="E223" s="6"/>
+      <c r="F223" s="6"/>
+      <c r="G223" s="6"/>
       <c r="H223" s="2"/>
     </row>
     <row r="224">
       <c r="A224" s="2"/>
-      <c r="B224" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 15</t>
-        </is>
-      </c>
-      <c r="C224" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Age of Jackson</t>
-        </is>
-      </c>
-      <c r="D224" s="16"/>
-      <c r="E224" s="16"/>
-      <c r="F224" s="16"/>
-      <c r="G224" s="17"/>
+      <c r="B224" s="2"/>
+      <c r="C224" s="2"/>
+      <c r="D224" s="2"/>
+      <c r="E224" s="2"/>
+      <c r="F224" s="2"/>
+      <c r="G224" s="2"/>
       <c r="H224" s="2"/>
     </row>
     <row r="225">
       <c r="A225" s="2"/>
-      <c r="B225" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C225" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The Age of Jackson</t>
-        </is>
-      </c>
-      <c r="D225" s="5"/>
-      <c r="E225" s="6"/>
-      <c r="F225" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.6.6, 8.8.1, 8.10.2, 8.4.3, 8.9.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G225" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did Andrew Jackson's presidency expand democracy for some Americans while increasing conflict over power, money, and rights?</t>
-        </is>
-      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 15</t>
+        </is>
+      </c>
+      <c r="C225" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Age of Jackson</t>
+        </is>
+      </c>
+      <c r="D225" s="16"/>
+      <c r="E225" s="16"/>
+      <c r="F225" s="16"/>
+      <c r="G225" s="17"/>
       <c r="H225" s="2"/>
     </row>
     <row r="226">
       <c r="A226" s="2"/>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C226" s="5"/>
-      <c r="D226" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C226" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Age of Jackson</t>
+        </is>
+      </c>
+      <c r="D226" s="5"/>
       <c r="E226" s="6"/>
-      <c r="F226" s="6"/>
-      <c r="G226" s="6"/>
+      <c r="F226" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.6.6, 8.8.1, 8.10.2, 8.4.3, 8.9.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G226" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Andrew Jackson's presidency expand democracy for some Americans while increasing conflict over power, money, and rights?</t>
+        </is>
+      </c>
       <c r="H226" s="2"/>
     </row>
     <row r="227">
       <c r="A227" s="2"/>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C227" s="5"/>
-      <c r="D227" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Jackson Wins the Presidency</t>
+      <c r="D227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E227" s="6"/>
@@ -4700,7 +4700,7 @@
       <c r="C228" s="5"/>
       <c r="D228" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Political Conflict and Economic Crisis</t>
+          <t xml:space="preserve">eText: Jackson Wins the Presidency</t>
         </is>
       </c>
       <c r="E228" s="6"/>
@@ -4712,53 +4712,53 @@
       <c r="A229" s="2"/>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C229" s="5"/>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Andrew Jackson and the Age of Jackson</t>
+          <t xml:space="preserve">eText: Political Conflict and Economic Crisis</t>
         </is>
       </c>
       <c r="E229" s="6"/>
       <c r="F229" s="6"/>
-      <c r="G229" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G229" s="6"/>
       <c r="H229" s="2"/>
     </row>
     <row r="230">
       <c r="A230" s="2"/>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C230" s="5"/>
-      <c r="D230" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D230" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Andrew Jackson and the Age of Jackson</t>
         </is>
       </c>
       <c r="E230" s="6"/>
       <c r="F230" s="6"/>
-      <c r="G230" s="6"/>
+      <c r="G230" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H230" s="2"/>
     </row>
     <row r="231">
       <c r="A231" s="2"/>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C231" s="5"/>
-      <c r="D231" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Timeline: Changing Voting Rights in Early America</t>
+      <c r="D231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E231" s="6"/>
@@ -4776,7 +4776,7 @@
       <c r="C232" s="5"/>
       <c r="D232" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Political Parties in the Age of Jackson</t>
+          <t xml:space="preserve">Interactive Timeline: Changing Voting Rights in Early America</t>
         </is>
       </c>
       <c r="E232" s="6"/>
@@ -4794,7 +4794,7 @@
       <c r="C233" s="5"/>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Tariffs and Trade</t>
+          <t xml:space="preserve">Interactive Chart: Political Parties in the Age of Jackson</t>
         </is>
       </c>
       <c r="E233" s="6"/>
@@ -4812,7 +4812,7 @@
       <c r="C234" s="5"/>
       <c r="D234" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Disagreements Over the Bank</t>
+          <t xml:space="preserve">Interactive Map: Tariffs and Trade</t>
         </is>
       </c>
       <c r="E234" s="6"/>
@@ -4824,22 +4824,18 @@
       <c r="A235" s="2"/>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C235" s="5"/>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Chart: Disagreements Over the Bank</t>
         </is>
       </c>
       <c r="E235" s="6"/>
       <c r="F235" s="6"/>
-      <c r="G235" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G235" s="6"/>
       <c r="H235" s="2"/>
     </row>
     <row r="236">
@@ -4852,14 +4848,14 @@
       <c r="C236" s="5"/>
       <c r="D236" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: Old Hickory Would Not Back Down</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E236" s="6"/>
       <c r="F236" s="6"/>
       <c r="G236" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">drag-and-drop</t>
+          <t xml:space="preserve">6 questions</t>
         </is>
       </c>
       <c r="H236" s="2"/>
@@ -4868,143 +4864,147 @@
       <c r="A237" s="2"/>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C237" s="5"/>
-      <c r="D237" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D237" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Old Hickory Would Not Back Down</t>
         </is>
       </c>
       <c r="E237" s="6"/>
       <c r="F237" s="6"/>
-      <c r="G237" s="6"/>
+      <c r="G237" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drag-and-drop</t>
+        </is>
+      </c>
       <c r="H237" s="2"/>
     </row>
     <row r="238">
       <c r="A238" s="2"/>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C238" s="5"/>
-      <c r="D238" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: The Age of Jackson</t>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E238" s="6"/>
       <c r="F238" s="6"/>
-      <c r="G238" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G238" s="6"/>
       <c r="H238" s="2"/>
     </row>
     <row r="239">
       <c r="A239" s="2"/>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C239" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Age of Jackson</t>
-        </is>
-      </c>
-      <c r="D239" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C239" s="5"/>
+      <c r="D239" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: The Age of Jackson</t>
+        </is>
+      </c>
       <c r="E239" s="6"/>
       <c r="F239" s="6"/>
-      <c r="G239" s="6"/>
+      <c r="G239" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H239" s="2"/>
     </row>
     <row r="240">
       <c r="A240" s="2"/>
-      <c r="B240" s="2"/>
-      <c r="C240" s="2"/>
-      <c r="D240" s="2"/>
-      <c r="E240" s="2"/>
-      <c r="F240" s="2"/>
-      <c r="G240" s="2"/>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C240" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Age of Jackson</t>
+        </is>
+      </c>
+      <c r="D240" s="5"/>
+      <c r="E240" s="6"/>
+      <c r="F240" s="6"/>
+      <c r="G240" s="6"/>
       <c r="H240" s="2"/>
     </row>
     <row r="241">
       <c r="A241" s="2"/>
-      <c r="B241" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 16</t>
-        </is>
-      </c>
-      <c r="C241" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">American Indians &amp; Westward Movement</t>
-        </is>
-      </c>
-      <c r="D241" s="16"/>
-      <c r="E241" s="16"/>
-      <c r="F241" s="16"/>
-      <c r="G241" s="17"/>
+      <c r="B241" s="2"/>
+      <c r="C241" s="2"/>
+      <c r="D241" s="2"/>
+      <c r="E241" s="2"/>
+      <c r="F241" s="2"/>
+      <c r="G241" s="2"/>
       <c r="H241" s="2"/>
     </row>
     <row r="242">
       <c r="A242" s="2"/>
-      <c r="B242" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C242" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | American Indians &amp; Westward Movement</t>
-        </is>
-      </c>
-      <c r="D242" s="5"/>
-      <c r="E242" s="6"/>
-      <c r="F242" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.8.1, 8.8.2, 8.12.2, 8.6.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G242" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did westward expansion affect American Indian nations and settlers, and what happens when law on paper does not match power in practice?</t>
-        </is>
-      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 16</t>
+        </is>
+      </c>
+      <c r="C242" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">American Indians &amp; Westward Movement</t>
+        </is>
+      </c>
+      <c r="D242" s="16"/>
+      <c r="E242" s="16"/>
+      <c r="F242" s="16"/>
+      <c r="G242" s="17"/>
       <c r="H242" s="2"/>
     </row>
     <row r="243">
       <c r="A243" s="2"/>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C243" s="5"/>
-      <c r="D243" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C243" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | American Indians &amp; Westward Movement</t>
+        </is>
+      </c>
+      <c r="D243" s="5"/>
       <c r="E243" s="6"/>
-      <c r="F243" s="6"/>
-      <c r="G243" s="6"/>
+      <c r="F243" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.8.1, 8.8.2, 8.12.2, 8.6.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G243" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did westward expansion affect American Indian nations and settlers, and what happens when law on paper does not match power in practice?</t>
+        </is>
+      </c>
       <c r="H243" s="2"/>
     </row>
     <row r="244">
       <c r="A244" s="2"/>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C244" s="5"/>
-      <c r="D244" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Conflict with American Indians</t>
+      <c r="D244" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E244" s="6"/>
@@ -5022,7 +5022,7 @@
       <c r="C245" s="5"/>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Westward Movement</t>
+          <t xml:space="preserve">eText: Conflict with American Indians</t>
         </is>
       </c>
       <c r="E245" s="6"/>
@@ -5034,53 +5034,53 @@
       <c r="A246" s="2"/>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C246" s="5"/>
       <c r="D246" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Removal, Law, and Westward Movement</t>
+          <t xml:space="preserve">eText: Westward Movement</t>
         </is>
       </c>
       <c r="E246" s="6"/>
       <c r="F246" s="6"/>
-      <c r="G246" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G246" s="6"/>
       <c r="H246" s="2"/>
     </row>
     <row r="247">
       <c r="A247" s="2"/>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C247" s="5"/>
-      <c r="D247" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D247" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Removal, Law, and Westward Movement</t>
         </is>
       </c>
       <c r="E247" s="6"/>
       <c r="F247" s="6"/>
-      <c r="G247" s="6"/>
+      <c r="G247" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H247" s="2"/>
     </row>
     <row r="248">
       <c r="A248" s="2"/>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C248" s="5"/>
-      <c r="D248" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Map: Selected Native American Groups</t>
+      <c r="D248" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E248" s="6"/>
@@ -5098,7 +5098,7 @@
       <c r="C249" s="5"/>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: The Trail of Tears</t>
+          <t xml:space="preserve">Interactive Map: Selected Native American Groups</t>
         </is>
       </c>
       <c r="E249" s="6"/>
@@ -5116,7 +5116,7 @@
       <c r="C250" s="5"/>
       <c r="D250" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: New Transportation Methods</t>
+          <t xml:space="preserve">Interactive Map: The Trail of Tears</t>
         </is>
       </c>
       <c r="E250" s="6"/>
@@ -5134,7 +5134,7 @@
       <c r="C251" s="5"/>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: New Technology: The Steamboat</t>
+          <t xml:space="preserve">Interactive Gallery: New Transportation Methods</t>
         </is>
       </c>
       <c r="E251" s="6"/>
@@ -5146,22 +5146,18 @@
       <c r="A252" s="2"/>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C252" s="5"/>
       <c r="D252" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Gallery: New Technology: The Steamboat</t>
         </is>
       </c>
       <c r="E252" s="6"/>
       <c r="F252" s="6"/>
-      <c r="G252" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G252" s="6"/>
       <c r="H252" s="2"/>
     </row>
     <row r="253">
@@ -5174,14 +5170,14 @@
       <c r="C253" s="5"/>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Cherokee Won, Then Lost It All</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E253" s="6"/>
       <c r="F253" s="6"/>
       <c r="G253" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">drag-and-drop</t>
+          <t xml:space="preserve">6 questions</t>
         </is>
       </c>
       <c r="H253" s="2"/>
@@ -5190,143 +5186,147 @@
       <c r="A254" s="2"/>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C254" s="5"/>
-      <c r="D254" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D254" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Cherokee Won, Then Lost It All</t>
         </is>
       </c>
       <c r="E254" s="6"/>
       <c r="F254" s="6"/>
-      <c r="G254" s="6"/>
+      <c r="G254" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drag-and-drop</t>
+        </is>
+      </c>
       <c r="H254" s="2"/>
     </row>
     <row r="255">
       <c r="A255" s="2"/>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C255" s="5"/>
-      <c r="D255" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: American Indians &amp; Westward Movement</t>
+      <c r="D255" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E255" s="6"/>
       <c r="F255" s="6"/>
-      <c r="G255" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G255" s="6"/>
       <c r="H255" s="2"/>
     </row>
     <row r="256">
       <c r="A256" s="2"/>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C256" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | American Indians &amp; Westward Movement</t>
-        </is>
-      </c>
-      <c r="D256" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C256" s="5"/>
+      <c r="D256" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: American Indians &amp; Westward Movement</t>
+        </is>
+      </c>
       <c r="E256" s="6"/>
       <c r="F256" s="6"/>
-      <c r="G256" s="6"/>
+      <c r="G256" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H256" s="2"/>
     </row>
     <row r="257">
       <c r="A257" s="2"/>
-      <c r="B257" s="2"/>
-      <c r="C257" s="2"/>
-      <c r="D257" s="2"/>
-      <c r="E257" s="2"/>
-      <c r="F257" s="2"/>
-      <c r="G257" s="2"/>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C257" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | American Indians &amp; Westward Movement</t>
+        </is>
+      </c>
+      <c r="D257" s="5"/>
+      <c r="E257" s="6"/>
+      <c r="F257" s="6"/>
+      <c r="G257" s="6"/>
       <c r="H257" s="2"/>
     </row>
     <row r="258">
       <c r="A258" s="2"/>
-      <c r="B258" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 17</t>
-        </is>
-      </c>
-      <c r="C258" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Settling Oregon &amp; Independence for Texas</t>
-        </is>
-      </c>
-      <c r="D258" s="16"/>
-      <c r="E258" s="16"/>
-      <c r="F258" s="16"/>
-      <c r="G258" s="17"/>
+      <c r="B258" s="2"/>
+      <c r="C258" s="2"/>
+      <c r="D258" s="2"/>
+      <c r="E258" s="2"/>
+      <c r="F258" s="2"/>
+      <c r="G258" s="2"/>
       <c r="H258" s="2"/>
     </row>
     <row r="259">
       <c r="A259" s="2"/>
-      <c r="B259" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C259" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Settling Oregon &amp; Independence for Texas</t>
-        </is>
-      </c>
-      <c r="D259" s="5"/>
-      <c r="E259" s="6"/>
-      <c r="F259" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.8.2, 8.8.3, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G259" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Why did Americans move into Oregon and Texas, and how did settlement in the West create new conflicts over land, independence, and annexation?</t>
-        </is>
-      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 17</t>
+        </is>
+      </c>
+      <c r="C259" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Settling Oregon &amp; Independence for Texas</t>
+        </is>
+      </c>
+      <c r="D259" s="16"/>
+      <c r="E259" s="16"/>
+      <c r="F259" s="16"/>
+      <c r="G259" s="17"/>
       <c r="H259" s="2"/>
     </row>
     <row r="260">
       <c r="A260" s="2"/>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C260" s="5"/>
-      <c r="D260" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C260" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Settling Oregon &amp; Independence for Texas</t>
+        </is>
+      </c>
+      <c r="D260" s="5"/>
       <c r="E260" s="6"/>
-      <c r="F260" s="6"/>
-      <c r="G260" s="6"/>
+      <c r="F260" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.8.2, 8.8.3, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G260" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why did Americans move into Oregon and Texas, and how did settlement in the West create new conflicts over land, independence, and annexation?</t>
+        </is>
+      </c>
       <c r="H260" s="2"/>
     </row>
     <row r="261">
       <c r="A261" s="2"/>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C261" s="5"/>
-      <c r="D261" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Settling Oregon Country</t>
+      <c r="D261" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E261" s="6"/>
@@ -5344,7 +5344,7 @@
       <c r="C262" s="5"/>
       <c r="D262" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: New Spain and Independence for Texas</t>
+          <t xml:space="preserve">eText: Settling Oregon Country</t>
         </is>
       </c>
       <c r="E262" s="6"/>
@@ -5356,53 +5356,53 @@
       <c r="A263" s="2"/>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C263" s="5"/>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Oregon, Texas, and Westward Settlement</t>
+          <t xml:space="preserve">eText: New Spain and Independence for Texas</t>
         </is>
       </c>
       <c r="E263" s="6"/>
       <c r="F263" s="6"/>
-      <c r="G263" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G263" s="6"/>
       <c r="H263" s="2"/>
     </row>
     <row r="264">
       <c r="A264" s="2"/>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C264" s="5"/>
-      <c r="D264" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D264" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Oregon, Texas, and Westward Settlement</t>
         </is>
       </c>
       <c r="E264" s="6"/>
       <c r="F264" s="6"/>
-      <c r="G264" s="6"/>
+      <c r="G264" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H264" s="2"/>
     </row>
     <row r="265">
       <c r="A265" s="2"/>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C265" s="5"/>
-      <c r="D265" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Map: Trails West</t>
+      <c r="D265" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E265" s="6"/>
@@ -5420,7 +5420,7 @@
       <c r="C266" s="5"/>
       <c r="D266" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: Life on the Oregon Trail</t>
+          <t xml:space="preserve">Interactive Map: Trails West</t>
         </is>
       </c>
       <c r="E266" s="6"/>
@@ -5438,7 +5438,7 @@
       <c r="C267" s="5"/>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Texas and the Southwest</t>
+          <t xml:space="preserve">Interactive Gallery: Life on the Oregon Trail</t>
         </is>
       </c>
       <c r="E267" s="6"/>
@@ -5456,7 +5456,7 @@
       <c r="C268" s="5"/>
       <c r="D268" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Timeline: Independence for Texas</t>
+          <t xml:space="preserve">Interactive Map: Texas and the Southwest</t>
         </is>
       </c>
       <c r="E268" s="6"/>
@@ -5468,22 +5468,18 @@
       <c r="A269" s="2"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C269" s="5"/>
       <c r="D269" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Timeline: Independence for Texas</t>
         </is>
       </c>
       <c r="E269" s="6"/>
       <c r="F269" s="6"/>
-      <c r="G269" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G269" s="6"/>
       <c r="H269" s="2"/>
     </row>
     <row r="270">
@@ -5496,25 +5492,29 @@
       <c r="C270" s="5"/>
       <c r="D270" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: Texas Was Its Own Country</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E270" s="6"/>
       <c r="F270" s="6"/>
-      <c r="G270" s="6"/>
+      <c r="G270" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H270" s="2"/>
     </row>
     <row r="271">
       <c r="A271" s="2"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C271" s="5"/>
-      <c r="D271" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D271" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Texas Was Its Own Country</t>
         </is>
       </c>
       <c r="E271" s="6"/>
@@ -5526,125 +5526,125 @@
       <c r="A272" s="2"/>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C272" s="5"/>
-      <c r="D272" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Settling Oregon &amp; Independence for Texas</t>
+      <c r="D272" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E272" s="6"/>
       <c r="F272" s="6"/>
-      <c r="G272" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G272" s="6"/>
       <c r="H272" s="2"/>
     </row>
     <row r="273">
       <c r="A273" s="2"/>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C273" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Settling Oregon &amp; Independence for Texas</t>
-        </is>
-      </c>
-      <c r="D273" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C273" s="5"/>
+      <c r="D273" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Settling Oregon &amp; Independence for Texas</t>
+        </is>
+      </c>
       <c r="E273" s="6"/>
       <c r="F273" s="6"/>
-      <c r="G273" s="6"/>
+      <c r="G273" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H273" s="2"/>
     </row>
     <row r="274">
       <c r="A274" s="2"/>
-      <c r="B274" s="2"/>
-      <c r="C274" s="2"/>
-      <c r="D274" s="2"/>
-      <c r="E274" s="2"/>
-      <c r="F274" s="2"/>
-      <c r="G274" s="2"/>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C274" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Settling Oregon &amp; Independence for Texas</t>
+        </is>
+      </c>
+      <c r="D274" s="5"/>
+      <c r="E274" s="6"/>
+      <c r="F274" s="6"/>
+      <c r="G274" s="6"/>
       <c r="H274" s="2"/>
     </row>
     <row r="275">
       <c r="A275" s="2"/>
-      <c r="B275" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 18</t>
-        </is>
-      </c>
-      <c r="C275" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manifest Destiny in California &amp; the Southwest</t>
-        </is>
-      </c>
-      <c r="D275" s="16"/>
-      <c r="E275" s="16"/>
-      <c r="F275" s="16"/>
-      <c r="G275" s="17"/>
+      <c r="B275" s="2"/>
+      <c r="C275" s="2"/>
+      <c r="D275" s="2"/>
+      <c r="E275" s="2"/>
+      <c r="F275" s="2"/>
+      <c r="G275" s="2"/>
       <c r="H275" s="2"/>
     </row>
     <row r="276">
       <c r="A276" s="2"/>
-      <c r="B276" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C276" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Manifest Destiny in California &amp; the Southwest</t>
-        </is>
-      </c>
-      <c r="D276" s="5"/>
-      <c r="E276" s="6"/>
-      <c r="F276" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.5.2, 8.6.2, 8.8.1, 8.8.2, 8.8.4, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G276" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did Manifest Destiny and the Mexican-American War change California, the Southwest, and the United States?</t>
-        </is>
-      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 18</t>
+        </is>
+      </c>
+      <c r="C276" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manifest Destiny in California &amp; the Southwest</t>
+        </is>
+      </c>
+      <c r="D276" s="16"/>
+      <c r="E276" s="16"/>
+      <c r="F276" s="16"/>
+      <c r="G276" s="17"/>
       <c r="H276" s="2"/>
     </row>
     <row r="277">
       <c r="A277" s="2"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C277" s="5"/>
-      <c r="D277" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C277" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Manifest Destiny in California &amp; the Southwest</t>
+        </is>
+      </c>
+      <c r="D277" s="5"/>
       <c r="E277" s="6"/>
-      <c r="F277" s="6"/>
-      <c r="G277" s="6"/>
+      <c r="F277" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.5.2, 8.6.2, 8.8.1, 8.8.2, 8.8.4, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G277" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Manifest Destiny and the Mexican-American War change California, the Southwest, and the United States?</t>
+        </is>
+      </c>
       <c r="H277" s="2"/>
     </row>
     <row r="278">
       <c r="A278" s="2"/>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C278" s="5"/>
-      <c r="D278" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Manifest Destiny in California and the Southwest</t>
+      <c r="D278" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E278" s="6"/>
@@ -5656,53 +5656,53 @@
       <c r="A279" s="2"/>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C279" s="5"/>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Manifest Destiny and the Mexican-American War</t>
+          <t xml:space="preserve">eText: Manifest Destiny in California and the Southwest</t>
         </is>
       </c>
       <c r="E279" s="6"/>
       <c r="F279" s="6"/>
-      <c r="G279" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G279" s="6"/>
       <c r="H279" s="2"/>
     </row>
     <row r="280">
       <c r="A280" s="2"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C280" s="5"/>
-      <c r="D280" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D280" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Manifest Destiny and the Mexican-American War</t>
         </is>
       </c>
       <c r="E280" s="6"/>
       <c r="F280" s="6"/>
-      <c r="G280" s="6"/>
+      <c r="G280" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H280" s="2"/>
     </row>
     <row r="281">
       <c r="A281" s="2"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C281" s="5"/>
-      <c r="D281" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Map: The Growth of the West to 1860</t>
+      <c r="D281" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E281" s="6"/>
@@ -5720,7 +5720,7 @@
       <c r="C282" s="5"/>
       <c r="D282" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: The People of California</t>
+          <t xml:space="preserve">Interactive Map: The Growth of the West to 1860</t>
         </is>
       </c>
       <c r="E282" s="6"/>
@@ -5732,22 +5732,18 @@
       <c r="A283" s="2"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C283" s="5"/>
       <c r="D283" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Interactive Gallery: The People of California</t>
         </is>
       </c>
       <c r="E283" s="6"/>
       <c r="F283" s="6"/>
-      <c r="G283" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 questions</t>
-        </is>
-      </c>
+      <c r="G283" s="6"/>
       <c r="H283" s="2"/>
     </row>
     <row r="284">
@@ -5760,25 +5756,29 @@
       <c r="C284" s="5"/>
       <c r="D284" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Bear Flag Republic: It Bearly Lasted a Month</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E284" s="6"/>
       <c r="F284" s="6"/>
-      <c r="G284" s="6"/>
+      <c r="G284" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H284" s="2"/>
     </row>
     <row r="285">
       <c r="A285" s="2"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C285" s="5"/>
-      <c r="D285" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D285" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Bear Flag Republic: It Bearly Lasted a Month</t>
         </is>
       </c>
       <c r="E285" s="6"/>
@@ -5790,112 +5790,112 @@
       <c r="A286" s="2"/>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C286" s="5"/>
-      <c r="D286" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Manifest Destiny in California &amp; the Southwest</t>
+      <c r="D286" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E286" s="6"/>
       <c r="F286" s="6"/>
-      <c r="G286" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="G286" s="6"/>
       <c r="H286" s="2"/>
     </row>
     <row r="287">
       <c r="A287" s="2"/>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C287" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Manifest Destiny in California &amp; the Southwest</t>
-        </is>
-      </c>
-      <c r="D287" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C287" s="5"/>
+      <c r="D287" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Manifest Destiny in California &amp; the Southwest</t>
+        </is>
+      </c>
       <c r="E287" s="6"/>
       <c r="F287" s="6"/>
-      <c r="G287" s="6"/>
+      <c r="G287" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H287" s="2"/>
     </row>
     <row r="288">
       <c r="A288" s="2"/>
-      <c r="B288" s="2"/>
-      <c r="C288" s="2"/>
-      <c r="D288" s="2"/>
-      <c r="E288" s="2"/>
-      <c r="F288" s="2"/>
-      <c r="G288" s="2"/>
+      <c r="B288" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C288" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Manifest Destiny in California &amp; the Southwest</t>
+        </is>
+      </c>
+      <c r="D288" s="5"/>
+      <c r="E288" s="6"/>
+      <c r="F288" s="6"/>
+      <c r="G288" s="6"/>
       <c r="H288" s="2"/>
     </row>
     <row r="289">
       <c r="A289" s="2"/>
-      <c r="B289" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 19</t>
-        </is>
-      </c>
-      <c r="C289" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT - Current Events Connection  (Project)</t>
-        </is>
-      </c>
-      <c r="D289" s="16"/>
-      <c r="E289" s="16"/>
-      <c r="F289" s="16"/>
-      <c r="G289" s="17"/>
+      <c r="B289" s="2"/>
+      <c r="C289" s="2"/>
+      <c r="D289" s="2"/>
+      <c r="E289" s="2"/>
+      <c r="F289" s="2"/>
+      <c r="G289" s="2"/>
       <c r="H289" s="2"/>
     </row>
     <row r="290">
       <c r="A290" s="2"/>
-      <c r="B290" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C290" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT - Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D290" s="5"/>
-      <c r="E290" s="6"/>
-      <c r="F290" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS Course-specific social science content standards connected to the student's chosen topic | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.7, W.8.8, W.8.9, SL.8.4, SL.8.5 | ELD Part I A.3, Part I B.6, Part I B.7, Part I C.10, Part I C.11</t>
-        </is>
-      </c>
-      <c r="G290" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How can a current event help us understand patterns, conflicts, and choices from the past?</t>
-        </is>
-      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 19</t>
+        </is>
+      </c>
+      <c r="C290" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Current Events Connection  (Project)</t>
+        </is>
+      </c>
+      <c r="D290" s="16"/>
+      <c r="E290" s="16"/>
+      <c r="F290" s="16"/>
+      <c r="G290" s="17"/>
       <c r="H290" s="2"/>
     </row>
     <row r="291">
       <c r="A291" s="2"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C291" s="5"/>
-      <c r="D291" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C291" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT - Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D291" s="5"/>
       <c r="E291" s="6"/>
-      <c r="F291" s="6"/>
-      <c r="G291" s="6"/>
+      <c r="F291" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS Course-specific social science content standards connected to the student's chosen topic | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.7, W.8.8, W.8.9, SL.8.4, SL.8.5 | ELD Part I A.3, Part I B.6, Part I B.7, Part I C.10, Part I C.11</t>
+        </is>
+      </c>
+      <c r="G291" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How can a current event help us understand patterns, conflicts, and choices from the past?</t>
+        </is>
+      </c>
       <c r="H291" s="2"/>
     </row>
     <row r="292">
@@ -5908,7 +5908,7 @@
       <c r="C292" s="5"/>
       <c r="D292" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E292" s="6"/>
@@ -5926,7 +5926,7 @@
       <c r="C293" s="5"/>
       <c r="D293" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E293" s="6"/>
@@ -5938,15 +5938,15 @@
       <c r="A294" s="2"/>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C294" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D294" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C294" s="5"/>
+      <c r="D294" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E294" s="6"/>
       <c r="F294" s="6"/>
       <c r="G294" s="6"/>
@@ -5954,92 +5954,88 @@
     </row>
     <row r="295">
       <c r="A295" s="2"/>
-      <c r="B295" s="2"/>
-      <c r="C295" s="2"/>
-      <c r="D295" s="2"/>
-      <c r="E295" s="2"/>
-      <c r="F295" s="2"/>
-      <c r="G295" s="2"/>
+      <c r="B295" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C295" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D295" s="5"/>
+      <c r="E295" s="6"/>
+      <c r="F295" s="6"/>
+      <c r="G295" s="6"/>
       <c r="H295" s="2"/>
     </row>
     <row r="296">
       <c r="A296" s="2"/>
-      <c r="B296" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 20</t>
-        </is>
-      </c>
-      <c r="C296" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Study Guide &amp; Final Exam  (Exam)</t>
-        </is>
-      </c>
-      <c r="D296" s="16"/>
-      <c r="E296" s="16"/>
-      <c r="F296" s="16"/>
-      <c r="G296" s="17"/>
+      <c r="B296" s="2"/>
+      <c r="C296" s="2"/>
+      <c r="D296" s="2"/>
+      <c r="E296" s="2"/>
+      <c r="F296" s="2"/>
+      <c r="G296" s="2"/>
       <c r="H296" s="2"/>
     </row>
     <row r="297">
       <c r="A297" s="2"/>
-      <c r="B297" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C297" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Study Guide &amp; Final Exam</t>
-        </is>
-      </c>
-      <c r="D297" s="5"/>
-      <c r="E297" s="6"/>
-      <c r="F297" s="6"/>
-      <c r="G297" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Semester 1 review and final exam</t>
-        </is>
-      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 20</t>
+        </is>
+      </c>
+      <c r="C297" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study Guide &amp; Final Exam  (Exam)</t>
+        </is>
+      </c>
+      <c r="D297" s="16"/>
+      <c r="E297" s="16"/>
+      <c r="F297" s="16"/>
+      <c r="G297" s="17"/>
       <c r="H297" s="2"/>
     </row>
     <row r="298">
       <c r="A298" s="2"/>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C298" s="5"/>
-      <c r="D298" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Study Guide and Final Exam</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C298" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D298" s="5"/>
       <c r="E298" s="6"/>
       <c r="F298" s="6"/>
-      <c r="G298" s="6"/>
+      <c r="G298" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semester 1 review and final exam</t>
+        </is>
+      </c>
       <c r="H298" s="2"/>
     </row>
     <row r="299">
       <c r="A299" s="2"/>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C299" s="5"/>
-      <c r="D299" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20.1 | Semester 1 Final Exam Study Guide</t>
+      <c r="D299" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study Guide and Final Exam</t>
         </is>
       </c>
       <c r="E299" s="6"/>
       <c r="F299" s="6"/>
-      <c r="G299" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Download the study guide, answer the questions in your own words, and study from your answers before the final exam. Download: US History 8-1 Final Exam Study Guide.docx</t>
-        </is>
-      </c>
+      <c r="G299" s="6"/>
       <c r="H299" s="2"/>
     </row>
     <row r="300">
@@ -6052,14 +6048,14 @@
       <c r="C300" s="5"/>
       <c r="D300" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">20.2 | Semester 1 Final Exam (Midterm)</t>
+          <t xml:space="preserve">20.1 | Semester 1 Final Exam Study Guide</t>
         </is>
       </c>
       <c r="E300" s="6"/>
       <c r="F300" s="6"/>
       <c r="G300" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your teacher will tell you when and where to complete the Semester 1 Final Exam. This may also be called the midterm.</t>
+          <t xml:space="preserve">Download the study guide, answer the questions in your own words, and study from your answers before the final exam. Download: US History 8-1 Final Exam Study Guide.docx</t>
         </is>
       </c>
       <c r="H300" s="2"/>
@@ -6068,73 +6064,95 @@
       <c r="A301" s="2"/>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Page</t>
         </is>
       </c>
       <c r="C301" s="5"/>
-      <c r="D301" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
+      <c r="D301" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20.2 | Semester 1 Final Exam (Midterm)</t>
         </is>
       </c>
       <c r="E301" s="6"/>
       <c r="F301" s="6"/>
-      <c r="G301" s="6"/>
+      <c r="G301" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Your teacher will tell you when and where to complete the Semester 1 Final Exam. This may also be called the midterm.</t>
+        </is>
+      </c>
       <c r="H301" s="2"/>
     </row>
     <row r="302">
       <c r="A302" s="2"/>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resource</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C302" s="5"/>
-      <c r="D302" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Printable study guide Word document</t>
+      <c r="D302" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
         </is>
       </c>
       <c r="E302" s="6"/>
       <c r="F302" s="6"/>
-      <c r="G302" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">course_planning/content/8-1/module-20-assets/US-History-8-1-Final-Exam-Study-Guide.docx</t>
-        </is>
-      </c>
+      <c r="G302" s="6"/>
       <c r="H302" s="2"/>
     </row>
     <row r="303">
       <c r="A303" s="2"/>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C303" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
-        </is>
-      </c>
-      <c r="D303" s="5"/>
+          <t xml:space="preserve">Resource</t>
+        </is>
+      </c>
+      <c r="C303" s="5"/>
+      <c r="D303" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable study guide Word document</t>
+        </is>
+      </c>
       <c r="E303" s="6"/>
       <c r="F303" s="6"/>
       <c r="G303" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module only contains review directions and the downloadable study guide.</t>
+          <t xml:space="preserve">course_planning/content/8-1/module-20-assets/US-History-8-1-Final-Exam-Study-Guide.docx</t>
         </is>
       </c>
       <c r="H303" s="2"/>
     </row>
     <row r="304">
       <c r="A304" s="2"/>
-      <c r="B304" s="2"/>
-      <c r="C304" s="2"/>
-      <c r="D304" s="2"/>
-      <c r="E304" s="2"/>
-      <c r="F304" s="2"/>
-      <c r="G304" s="2"/>
+      <c r="B304" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C304" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D304" s="5"/>
+      <c r="E304" s="6"/>
+      <c r="F304" s="6"/>
+      <c r="G304" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module only contains review directions and the downloadable study guide.</t>
+        </is>
+      </c>
       <c r="H304" s="2"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="2"/>
+      <c r="B305" s="2"/>
+      <c r="C305" s="2"/>
+      <c r="D305" s="2"/>
+      <c r="E305" s="2"/>
+      <c r="F305" s="2"/>
+      <c r="G305" s="2"/>
+      <c r="H305" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -6148,18 +6166,18 @@
     <mergeCell ref="C95:G95"/>
     <mergeCell ref="C108:G108"/>
     <mergeCell ref="C125:G125"/>
-    <mergeCell ref="C140:G140"/>
-    <mergeCell ref="C157:G157"/>
-    <mergeCell ref="C173:G173"/>
-    <mergeCell ref="C188:G188"/>
-    <mergeCell ref="C196:G196"/>
-    <mergeCell ref="C210:G210"/>
-    <mergeCell ref="C224:G224"/>
-    <mergeCell ref="C241:G241"/>
-    <mergeCell ref="C258:G258"/>
-    <mergeCell ref="C275:G275"/>
-    <mergeCell ref="C289:G289"/>
-    <mergeCell ref="C296:G296"/>
+    <mergeCell ref="C141:G141"/>
+    <mergeCell ref="C158:G158"/>
+    <mergeCell ref="C174:G174"/>
+    <mergeCell ref="C189:G189"/>
+    <mergeCell ref="C197:G197"/>
+    <mergeCell ref="C211:G211"/>
+    <mergeCell ref="C225:G225"/>
+    <mergeCell ref="C242:G242"/>
+    <mergeCell ref="C259:G259"/>
+    <mergeCell ref="C276:G276"/>
+    <mergeCell ref="C290:G290"/>
+    <mergeCell ref="C297:G297"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify Module 8 around DBQ
</commit_message>
<xml_diff>
--- a/exports/US History 8-1 - Course Outline.xlsx
+++ b/exports/US History 8-1 - Course Outline.xlsx
@@ -2888,7 +2888,7 @@
       <c r="C132" s="5"/>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biography: Alexander Hamilton</t>
+          <t xml:space="preserve">8.3.1 | DBQ: Constitutional Debates</t>
         </is>
       </c>
       <c r="E132" s="6"/>
@@ -2900,31 +2900,35 @@
       <c r="A133" s="2"/>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C133" s="5"/>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Primary Source: United States Constitution</t>
+          <t xml:space="preserve">Stranger Than Fiction: Graded a 'C,' Then He Changed the Constitution</t>
         </is>
       </c>
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
-      <c r="G133" s="6"/>
+      <c r="G133" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 questions</t>
+        </is>
+      </c>
       <c r="H133" s="2"/>
     </row>
     <row r="134">
       <c r="A134" s="2"/>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C134" s="5"/>
-      <c r="D134" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8.3.5 | DBQ: Constitutional Debates</t>
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E134" s="6"/>
@@ -2942,14 +2946,14 @@
       <c r="C135" s="5"/>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Ratification &amp; How the Constitution Works</t>
         </is>
       </c>
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
       <c r="G135" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H135" s="2"/>
@@ -2958,62 +2962,46 @@
       <c r="A136" s="2"/>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C136" s="5"/>
-      <c r="D136" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: Graded a 'C,' Then He Changed the Constitution</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Ratification &amp; How the Constitution Works</t>
+        </is>
+      </c>
+      <c r="D136" s="5"/>
       <c r="E136" s="6"/>
       <c r="F136" s="6"/>
-      <c r="G136" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 questions</t>
-        </is>
-      </c>
+      <c r="G136" s="6"/>
       <c r="H136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2"/>
-      <c r="B137" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C137" s="5"/>
-      <c r="D137" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E137" s="6"/>
-      <c r="F137" s="6"/>
-      <c r="G137" s="6"/>
+      <c r="B137" s="2"/>
+      <c r="C137" s="2"/>
+      <c r="D137" s="2"/>
+      <c r="E137" s="2"/>
+      <c r="F137" s="2"/>
+      <c r="G137" s="2"/>
       <c r="H137" s="2"/>
     </row>
     <row r="138">
       <c r="A138" s="2"/>
-      <c r="B138" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C138" s="5"/>
-      <c r="D138" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Ratification &amp; How the Constitution Works</t>
-        </is>
-      </c>
-      <c r="E138" s="6"/>
-      <c r="F138" s="6"/>
-      <c r="G138" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 9</t>
+        </is>
+      </c>
+      <c r="C138" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Federalism &amp; Citizenship</t>
+        </is>
+      </c>
+      <c r="D138" s="16"/>
+      <c r="E138" s="16"/>
+      <c r="F138" s="16"/>
+      <c r="G138" s="17"/>
       <c r="H138" s="2"/>
     </row>
     <row r="139">
@@ -3025,98 +3013,110 @@
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Ratification &amp; How the Constitution Works</t>
+          <t xml:space="preserve">Overview | Federalism &amp; Citizenship</t>
         </is>
       </c>
       <c r="D139" s="5"/>
       <c r="E139" s="6"/>
-      <c r="F139" s="6"/>
-      <c r="G139" s="6"/>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.2.3, 8.2.6, 8.3.1, 8.3.6 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+        </is>
+      </c>
+      <c r="G139" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How does the Constitution divide power between national and state governments, and what rights and responsibilities come with U.S. citizenship?</t>
+        </is>
+      </c>
       <c r="H139" s="2"/>
     </row>
     <row r="140">
       <c r="A140" s="2"/>
-      <c r="B140" s="2"/>
-      <c r="C140" s="2"/>
-      <c r="D140" s="2"/>
-      <c r="E140" s="2"/>
-      <c r="F140" s="2"/>
-      <c r="G140" s="2"/>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C140" s="5"/>
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E140" s="6"/>
+      <c r="F140" s="6"/>
+      <c r="G140" s="6"/>
       <c r="H140" s="2"/>
     </row>
     <row r="141">
       <c r="A141" s="2"/>
-      <c r="B141" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 9</t>
-        </is>
-      </c>
-      <c r="C141" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Federalism &amp; Citizenship</t>
-        </is>
-      </c>
-      <c r="D141" s="16"/>
-      <c r="E141" s="16"/>
-      <c r="F141" s="16"/>
-      <c r="G141" s="17"/>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C141" s="5"/>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Federalism and Amendments</t>
+        </is>
+      </c>
+      <c r="E141" s="6"/>
+      <c r="F141" s="6"/>
+      <c r="G141" s="6"/>
       <c r="H141" s="2"/>
     </row>
     <row r="142">
       <c r="A142" s="2"/>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Federalism &amp; Citizenship</t>
-        </is>
-      </c>
-      <c r="D142" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C142" s="5"/>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Citizens' Rights and Responsibilities</t>
+        </is>
+      </c>
       <c r="E142" s="6"/>
-      <c r="F142" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.2.3, 8.2.6, 8.3.1, 8.3.6 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
-        </is>
-      </c>
-      <c r="G142" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How does the Constitution divide power between national and state governments, and what rights and responsibilities come with U.S. citizenship?</t>
-        </is>
-      </c>
+      <c r="F142" s="6"/>
+      <c r="G142" s="6"/>
       <c r="H142" s="2"/>
     </row>
     <row r="143">
       <c r="A143" s="2"/>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C143" s="5"/>
-      <c r="D143" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Federalism and Citizenship</t>
         </is>
       </c>
       <c r="E143" s="6"/>
       <c r="F143" s="6"/>
-      <c r="G143" s="6"/>
+      <c r="G143" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H143" s="2"/>
     </row>
     <row r="144">
       <c r="A144" s="2"/>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C144" s="5"/>
-      <c r="D144" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Federalism and Amendments</t>
+      <c r="D144" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E144" s="6"/>
@@ -3134,7 +3134,7 @@
       <c r="C145" s="5"/>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Citizens' Rights and Responsibilities</t>
+          <t xml:space="preserve">Interactive Chart: Methods of Amending the Constitution</t>
         </is>
       </c>
       <c r="E145" s="6"/>
@@ -3146,35 +3146,31 @@
       <c r="A146" s="2"/>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C146" s="5"/>
       <c r="D146" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Federalism and Citizenship</t>
+          <t xml:space="preserve">Interactive Gallery: The First Amendment</t>
         </is>
       </c>
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
-      <c r="G146" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G146" s="6"/>
       <c r="H146" s="2"/>
     </row>
     <row r="147">
       <c r="A147" s="2"/>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C147" s="5"/>
-      <c r="D147" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Voting Responsibly</t>
         </is>
       </c>
       <c r="E147" s="6"/>
@@ -3192,7 +3188,7 @@
       <c r="C148" s="5"/>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Methods of Amending the Constitution</t>
+          <t xml:space="preserve">Interactive Chart: Civic Responsibility</t>
         </is>
       </c>
       <c r="E148" s="6"/>
@@ -3204,31 +3200,35 @@
       <c r="A149" s="2"/>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C149" s="5"/>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: The First Amendment</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E149" s="6"/>
       <c r="F149" s="6"/>
-      <c r="G149" s="6"/>
+      <c r="G149" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H149" s="2"/>
     </row>
     <row r="150">
       <c r="A150" s="2"/>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C150" s="5"/>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Voting Responsibly</t>
+          <t xml:space="preserve">Stranger Than Fiction: Old Enough to Fight, Too Young to Vote</t>
         </is>
       </c>
       <c r="E150" s="6"/>
@@ -3240,13 +3240,13 @@
       <c r="A151" s="2"/>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C151" s="5"/>
-      <c r="D151" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Chart: Civic Responsibility</t>
+      <c r="D151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E151" s="6"/>
@@ -3264,14 +3264,14 @@
       <c r="C152" s="5"/>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Federalism &amp; Citizenship</t>
         </is>
       </c>
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H152" s="2"/>
@@ -3280,15 +3280,15 @@
       <c r="A153" s="2"/>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C153" s="5"/>
-      <c r="D153" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: Old Enough to Fight, Too Young to Vote</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Federalism &amp; Citizenship</t>
+        </is>
+      </c>
+      <c r="D153" s="5"/>
       <c r="E153" s="6"/>
       <c r="F153" s="6"/>
       <c r="G153" s="6"/>
@@ -3296,42 +3296,30 @@
     </row>
     <row r="154">
       <c r="A154" s="2"/>
-      <c r="B154" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C154" s="5"/>
-      <c r="D154" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E154" s="6"/>
-      <c r="F154" s="6"/>
-      <c r="G154" s="6"/>
+      <c r="B154" s="2"/>
+      <c r="C154" s="2"/>
+      <c r="D154" s="2"/>
+      <c r="E154" s="2"/>
+      <c r="F154" s="2"/>
+      <c r="G154" s="2"/>
       <c r="H154" s="2"/>
     </row>
     <row r="155">
       <c r="A155" s="2"/>
-      <c r="B155" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C155" s="5"/>
-      <c r="D155" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Federalism &amp; Citizenship</t>
-        </is>
-      </c>
-      <c r="E155" s="6"/>
-      <c r="F155" s="6"/>
-      <c r="G155" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 10</t>
+        </is>
+      </c>
+      <c r="C155" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Washington's Presidency &amp; the Two-Party System</t>
+        </is>
+      </c>
+      <c r="D155" s="16"/>
+      <c r="E155" s="16"/>
+      <c r="F155" s="16"/>
+      <c r="G155" s="17"/>
       <c r="H155" s="2"/>
     </row>
     <row r="156">
@@ -3343,98 +3331,110 @@
       </c>
       <c r="C156" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Federalism &amp; Citizenship</t>
+          <t xml:space="preserve">Overview | Washington's Presidency &amp; the Two-Party System</t>
         </is>
       </c>
       <c r="D156" s="5"/>
       <c r="E156" s="6"/>
-      <c r="F156" s="6"/>
-      <c r="G156" s="6"/>
+      <c r="F156" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+        </is>
+      </c>
+      <c r="G156" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Washington shape the presidency, and why did political parties begin to form in the new republic?</t>
+        </is>
+      </c>
       <c r="H156" s="2"/>
     </row>
     <row r="157">
       <c r="A157" s="2"/>
-      <c r="B157" s="2"/>
-      <c r="C157" s="2"/>
-      <c r="D157" s="2"/>
-      <c r="E157" s="2"/>
-      <c r="F157" s="2"/>
-      <c r="G157" s="2"/>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C157" s="5"/>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E157" s="6"/>
+      <c r="F157" s="6"/>
+      <c r="G157" s="6"/>
       <c r="H157" s="2"/>
     </row>
     <row r="158">
       <c r="A158" s="2"/>
-      <c r="B158" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 10</t>
-        </is>
-      </c>
-      <c r="C158" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Washington's Presidency &amp; the Two-Party System</t>
-        </is>
-      </c>
-      <c r="D158" s="16"/>
-      <c r="E158" s="16"/>
-      <c r="F158" s="16"/>
-      <c r="G158" s="17"/>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C158" s="5"/>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Washington's Presidency</t>
+        </is>
+      </c>
+      <c r="E158" s="6"/>
+      <c r="F158" s="6"/>
+      <c r="G158" s="6"/>
       <c r="H158" s="2"/>
     </row>
     <row r="159">
       <c r="A159" s="2"/>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C159" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Washington's Presidency &amp; the Two-Party System</t>
-        </is>
-      </c>
-      <c r="D159" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C159" s="5"/>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: A Two-Party System Develops</t>
+        </is>
+      </c>
       <c r="E159" s="6"/>
-      <c r="F159" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.4, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
-        </is>
-      </c>
-      <c r="G159" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did Washington shape the presidency, and why did political parties begin to form in the new republic?</t>
-        </is>
-      </c>
+      <c r="F159" s="6"/>
+      <c r="G159" s="6"/>
       <c r="H159" s="2"/>
     </row>
     <row r="160">
       <c r="A160" s="2"/>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C160" s="5"/>
-      <c r="D160" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D160" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Washington's Presidency and First Political Parties</t>
         </is>
       </c>
       <c r="E160" s="6"/>
       <c r="F160" s="6"/>
-      <c r="G160" s="6"/>
+      <c r="G160" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H160" s="2"/>
     </row>
     <row r="161">
       <c r="A161" s="2"/>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C161" s="5"/>
-      <c r="D161" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Washington's Presidency</t>
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E161" s="6"/>
@@ -3452,7 +3452,7 @@
       <c r="C162" s="5"/>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: A Two-Party System Develops</t>
+          <t xml:space="preserve">Interactive Chart: A Controversial Tax</t>
         </is>
       </c>
       <c r="E162" s="6"/>
@@ -3464,35 +3464,31 @@
       <c r="A163" s="2"/>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C163" s="5"/>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Washington's Presidency and First Political Parties</t>
+          <t xml:space="preserve">Interactive Map: Foreign Affairs Under Washington</t>
         </is>
       </c>
       <c r="E163" s="6"/>
       <c r="F163" s="6"/>
-      <c r="G163" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G163" s="6"/>
       <c r="H163" s="2"/>
     </row>
     <row r="164">
       <c r="A164" s="2"/>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C164" s="5"/>
-      <c r="D164" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D164" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Early American Leaders</t>
         </is>
       </c>
       <c r="E164" s="6"/>
@@ -3504,49 +3500,57 @@
       <c r="A165" s="2"/>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C165" s="5"/>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: A Controversial Tax</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E165" s="6"/>
       <c r="F165" s="6"/>
-      <c r="G165" s="6"/>
+      <c r="G165" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H165" s="2"/>
     </row>
     <row r="166">
       <c r="A166" s="2"/>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C166" s="5"/>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Foreign Affairs Under Washington</t>
+          <t xml:space="preserve">Stranger Than Fiction: Would You Fight the Government Over Whiskey?</t>
         </is>
       </c>
       <c r="E166" s="6"/>
       <c r="F166" s="6"/>
-      <c r="G166" s="6"/>
+      <c r="G166" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drag-and-drop</t>
+        </is>
+      </c>
       <c r="H166" s="2"/>
     </row>
     <row r="167">
       <c r="A167" s="2"/>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C167" s="5"/>
-      <c r="D167" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Gallery: Early American Leaders</t>
+      <c r="D167" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E167" s="6"/>
@@ -3564,14 +3568,14 @@
       <c r="C168" s="5"/>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Washington's Presidency &amp; the Two-Party System</t>
         </is>
       </c>
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
       <c r="G168" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H168" s="2"/>
@@ -3580,62 +3584,46 @@
       <c r="A169" s="2"/>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C169" s="5"/>
-      <c r="D169" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: Would You Fight the Government Over Whiskey?</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Washington's Presidency &amp; the Two-Party System</t>
+        </is>
+      </c>
+      <c r="D169" s="5"/>
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
-      <c r="G169" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">drag-and-drop</t>
-        </is>
-      </c>
+      <c r="G169" s="6"/>
       <c r="H169" s="2"/>
     </row>
     <row r="170">
       <c r="A170" s="2"/>
-      <c r="B170" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C170" s="5"/>
-      <c r="D170" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E170" s="6"/>
-      <c r="F170" s="6"/>
-      <c r="G170" s="6"/>
+      <c r="B170" s="2"/>
+      <c r="C170" s="2"/>
+      <c r="D170" s="2"/>
+      <c r="E170" s="2"/>
+      <c r="F170" s="2"/>
+      <c r="G170" s="2"/>
       <c r="H170" s="2"/>
     </row>
     <row r="171">
       <c r="A171" s="2"/>
-      <c r="B171" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C171" s="5"/>
-      <c r="D171" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Washington's Presidency &amp; the Two-Party System</t>
-        </is>
-      </c>
-      <c r="E171" s="6"/>
-      <c r="F171" s="6"/>
-      <c r="G171" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 11</t>
+        </is>
+      </c>
+      <c r="C171" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adams, Jefferson &amp; a Changing Nation</t>
+        </is>
+      </c>
+      <c r="D171" s="16"/>
+      <c r="E171" s="16"/>
+      <c r="F171" s="16"/>
+      <c r="G171" s="17"/>
       <c r="H171" s="2"/>
     </row>
     <row r="172">
@@ -3647,98 +3635,110 @@
       </c>
       <c r="C172" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Washington's Presidency &amp; the Two-Party System</t>
+          <t xml:space="preserve">Overview | Adams, Jefferson &amp; a Changing Nation</t>
         </is>
       </c>
       <c r="D172" s="5"/>
       <c r="E172" s="6"/>
-      <c r="F172" s="6"/>
-      <c r="G172" s="6"/>
+      <c r="F172" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.4, 8.4.1, 8.5.2, 8.8.2, 8.8.4 | CCSS-ELA RH.1, RH.2, RH.4, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
+        </is>
+      </c>
+      <c r="G172" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did the presidencies of John Adams and Thomas Jefferson test the young nation's political ideas, rights, and expansion?</t>
+        </is>
+      </c>
       <c r="H172" s="2"/>
     </row>
     <row r="173">
       <c r="A173" s="2"/>
-      <c r="B173" s="2"/>
-      <c r="C173" s="2"/>
-      <c r="D173" s="2"/>
-      <c r="E173" s="2"/>
-      <c r="F173" s="2"/>
-      <c r="G173" s="2"/>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C173" s="5"/>
+      <c r="D173" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E173" s="6"/>
+      <c r="F173" s="6"/>
+      <c r="G173" s="6"/>
       <c r="H173" s="2"/>
     </row>
     <row r="174">
       <c r="A174" s="2"/>
-      <c r="B174" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 11</t>
-        </is>
-      </c>
-      <c r="C174" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adams, Jefferson &amp; a Changing Nation</t>
-        </is>
-      </c>
-      <c r="D174" s="16"/>
-      <c r="E174" s="16"/>
-      <c r="F174" s="16"/>
-      <c r="G174" s="17"/>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C174" s="5"/>
+      <c r="D174" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Presidents Adams and Jefferson</t>
+        </is>
+      </c>
+      <c r="E174" s="6"/>
+      <c r="F174" s="6"/>
+      <c r="G174" s="6"/>
       <c r="H174" s="2"/>
     </row>
     <row r="175">
       <c r="A175" s="2"/>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C175" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Adams, Jefferson &amp; a Changing Nation</t>
-        </is>
-      </c>
-      <c r="D175" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C175" s="5"/>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: A Changing Nation</t>
+        </is>
+      </c>
       <c r="E175" s="6"/>
-      <c r="F175" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.4, 8.4.1, 8.5.2, 8.8.2, 8.8.4 | CCSS-ELA RH.1, RH.2, RH.4, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b</t>
-        </is>
-      </c>
-      <c r="G175" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did the presidencies of John Adams and Thomas Jefferson test the young nation's political ideas, rights, and expansion?</t>
-        </is>
-      </c>
+      <c r="F175" s="6"/>
+      <c r="G175" s="6"/>
       <c r="H175" s="2"/>
     </row>
     <row r="176">
       <c r="A176" s="2"/>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C176" s="5"/>
-      <c r="D176" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D176" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Adams, Jefferson, and Expansion</t>
         </is>
       </c>
       <c r="E176" s="6"/>
       <c r="F176" s="6"/>
-      <c r="G176" s="6"/>
+      <c r="G176" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H176" s="2"/>
     </row>
     <row r="177">
       <c r="A177" s="2"/>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C177" s="5"/>
-      <c r="D177" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Presidents Adams and Jefferson</t>
+      <c r="D177" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E177" s="6"/>
@@ -3756,7 +3756,7 @@
       <c r="C178" s="5"/>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: A Changing Nation</t>
+          <t xml:space="preserve">Interactive Chart: Hamilton, Adams, or Jefferson?</t>
         </is>
       </c>
       <c r="E178" s="6"/>
@@ -3768,71 +3768,75 @@
       <c r="A179" s="2"/>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C179" s="5"/>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Adams, Jefferson, and Expansion</t>
+          <t xml:space="preserve">Interactive Map: Expansion and Exploration</t>
         </is>
       </c>
       <c r="E179" s="6"/>
       <c r="F179" s="6"/>
-      <c r="G179" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G179" s="6"/>
       <c r="H179" s="2"/>
     </row>
     <row r="180">
       <c r="A180" s="2"/>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C180" s="5"/>
-      <c r="D180" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E180" s="6"/>
       <c r="F180" s="6"/>
-      <c r="G180" s="6"/>
+      <c r="G180" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H180" s="2"/>
     </row>
     <row r="181">
       <c r="A181" s="2"/>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C181" s="5"/>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Hamilton, Adams, or Jefferson?</t>
+          <t xml:space="preserve">Stranger Than Fiction: Jefferson's Monster Map</t>
         </is>
       </c>
       <c r="E181" s="6"/>
       <c r="F181" s="6"/>
-      <c r="G181" s="6"/>
+      <c r="G181" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 questions</t>
+        </is>
+      </c>
       <c r="H181" s="2"/>
     </row>
     <row r="182">
       <c r="A182" s="2"/>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C182" s="5"/>
-      <c r="D182" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Map: Expansion and Exploration</t>
+      <c r="D182" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E182" s="6"/>
@@ -3850,14 +3854,14 @@
       <c r="C183" s="5"/>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Adams, Jefferson &amp; a Changing Nation</t>
         </is>
       </c>
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
       <c r="G183" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H183" s="2"/>
@@ -3866,62 +3870,46 @@
       <c r="A184" s="2"/>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C184" s="5"/>
-      <c r="D184" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: Jefferson's Monster Map</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Adams, Jefferson &amp; a Changing Nation</t>
+        </is>
+      </c>
+      <c r="D184" s="5"/>
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
-      <c r="G184" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 questions</t>
-        </is>
-      </c>
+      <c r="G184" s="6"/>
       <c r="H184" s="2"/>
     </row>
     <row r="185">
       <c r="A185" s="2"/>
-      <c r="B185" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C185" s="5"/>
-      <c r="D185" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E185" s="6"/>
-      <c r="F185" s="6"/>
-      <c r="G185" s="6"/>
+      <c r="B185" s="2"/>
+      <c r="C185" s="2"/>
+      <c r="D185" s="2"/>
+      <c r="E185" s="2"/>
+      <c r="F185" s="2"/>
+      <c r="G185" s="2"/>
       <c r="H185" s="2"/>
     </row>
     <row r="186">
       <c r="A186" s="2"/>
-      <c r="B186" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C186" s="5"/>
-      <c r="D186" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Adams, Jefferson &amp; a Changing Nation</t>
-        </is>
-      </c>
-      <c r="E186" s="6"/>
-      <c r="F186" s="6"/>
-      <c r="G186" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 12</t>
+        </is>
+      </c>
+      <c r="C186" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Dueling Leaders: Burr vs Hamilton  (Project)</t>
+        </is>
+      </c>
+      <c r="D186" s="16"/>
+      <c r="E186" s="16"/>
+      <c r="F186" s="16"/>
+      <c r="G186" s="17"/>
       <c r="H186" s="2"/>
     </row>
     <row r="187">
@@ -3933,67 +3921,79 @@
       </c>
       <c r="C187" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Adams, Jefferson &amp; a Changing Nation</t>
+          <t xml:space="preserve">Overview | PROJECT - Dueling Leaders: Burr vs Hamilton</t>
         </is>
       </c>
       <c r="D187" s="5"/>
       <c r="E187" s="6"/>
-      <c r="F187" s="6"/>
-      <c r="G187" s="6"/>
+      <c r="F187" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.9, WHST.1, WHST.4 | ELD Part I A.3, Part I B.6, Part I C.10, Part I C.11</t>
+        </is>
+      </c>
+      <c r="G187" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Should Aaron Burr have been found criminally responsible for Alexander Hamilton's death?</t>
+        </is>
+      </c>
       <c r="H187" s="2"/>
     </row>
     <row r="188">
       <c r="A188" s="2"/>
-      <c r="B188" s="2"/>
-      <c r="C188" s="2"/>
-      <c r="D188" s="2"/>
-      <c r="E188" s="2"/>
-      <c r="F188" s="2"/>
-      <c r="G188" s="2"/>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C188" s="5"/>
+      <c r="D188" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E188" s="6"/>
+      <c r="F188" s="6"/>
+      <c r="G188" s="6"/>
       <c r="H188" s="2"/>
     </row>
     <row r="189">
       <c r="A189" s="2"/>
-      <c r="B189" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 12</t>
-        </is>
-      </c>
-      <c r="C189" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT - Dueling Leaders: Burr vs Hamilton  (Project)</t>
-        </is>
-      </c>
-      <c r="D189" s="16"/>
-      <c r="E189" s="16"/>
-      <c r="F189" s="16"/>
-      <c r="G189" s="17"/>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C189" s="5"/>
+      <c r="D189" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Hamilton and Burr: The Duel That Became a Case File</t>
+        </is>
+      </c>
+      <c r="E189" s="6"/>
+      <c r="F189" s="6"/>
+      <c r="G189" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 check questions</t>
+        </is>
+      </c>
       <c r="H189" s="2"/>
     </row>
     <row r="190">
       <c r="A190" s="2"/>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C190" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT - Dueling Leaders: Burr vs Hamilton</t>
-        </is>
-      </c>
-      <c r="D190" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C190" s="5"/>
+      <c r="D190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E190" s="6"/>
-      <c r="F190" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.4, 8.3.5 | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.9, WHST.1, WHST.4 | ELD Part I A.3, Part I B.6, Part I C.10, Part I C.11</t>
-        </is>
-      </c>
-      <c r="G190" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Should Aaron Burr have been found criminally responsible for Alexander Hamilton's death?</t>
-        </is>
-      </c>
+      <c r="F190" s="6"/>
+      <c r="G190" s="6"/>
       <c r="H190" s="2"/>
     </row>
     <row r="191">
@@ -4006,7 +4006,7 @@
       <c r="C191" s="5"/>
       <c r="D191" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E191" s="6"/>
@@ -4018,58 +4018,46 @@
       <c r="A192" s="2"/>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C192" s="5"/>
-      <c r="D192" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Video: Hamilton and Burr: The Duel That Became a Case File</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C192" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Dueling Leaders: Burr vs Hamilton</t>
+        </is>
+      </c>
+      <c r="D192" s="5"/>
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
-      <c r="G192" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 check questions</t>
-        </is>
-      </c>
+      <c r="G192" s="6"/>
       <c r="H192" s="2"/>
     </row>
     <row r="193">
       <c r="A193" s="2"/>
-      <c r="B193" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C193" s="5"/>
-      <c r="D193" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E193" s="6"/>
-      <c r="F193" s="6"/>
-      <c r="G193" s="6"/>
+      <c r="B193" s="2"/>
+      <c r="C193" s="2"/>
+      <c r="D193" s="2"/>
+      <c r="E193" s="2"/>
+      <c r="F193" s="2"/>
+      <c r="G193" s="2"/>
       <c r="H193" s="2"/>
     </row>
     <row r="194">
       <c r="A194" s="2"/>
-      <c r="B194" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C194" s="5"/>
-      <c r="D194" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E194" s="6"/>
-      <c r="F194" s="6"/>
-      <c r="G194" s="6"/>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 13</t>
+        </is>
+      </c>
+      <c r="C194" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Madison &amp; the War of 1812</t>
+        </is>
+      </c>
+      <c r="D194" s="16"/>
+      <c r="E194" s="16"/>
+      <c r="F194" s="16"/>
+      <c r="G194" s="17"/>
       <c r="H194" s="2"/>
     </row>
     <row r="195">
@@ -4081,65 +4069,77 @@
       </c>
       <c r="C195" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Dueling Leaders: Burr vs Hamilton</t>
+          <t xml:space="preserve">Overview | Madison &amp; the War of 1812</t>
         </is>
       </c>
       <c r="D195" s="5"/>
       <c r="E195" s="6"/>
-      <c r="F195" s="6"/>
-      <c r="G195" s="6"/>
+      <c r="F195" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.5.1, 8.5.2, 8.5.3, 8.12.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G195" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why did the United States go to war with Britain in 1812, and how did the war change Americans' sense of national identity?</t>
+        </is>
+      </c>
       <c r="H195" s="2"/>
     </row>
     <row r="196">
       <c r="A196" s="2"/>
-      <c r="B196" s="2"/>
-      <c r="C196" s="2"/>
-      <c r="D196" s="2"/>
-      <c r="E196" s="2"/>
-      <c r="F196" s="2"/>
-      <c r="G196" s="2"/>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C196" s="5"/>
+      <c r="D196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E196" s="6"/>
+      <c r="F196" s="6"/>
+      <c r="G196" s="6"/>
       <c r="H196" s="2"/>
     </row>
     <row r="197">
       <c r="A197" s="2"/>
-      <c r="B197" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 13</t>
-        </is>
-      </c>
-      <c r="C197" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Madison &amp; the War of 1812</t>
-        </is>
-      </c>
-      <c r="D197" s="16"/>
-      <c r="E197" s="16"/>
-      <c r="F197" s="16"/>
-      <c r="G197" s="17"/>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C197" s="5"/>
+      <c r="D197" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Madison and the War of 1812</t>
+        </is>
+      </c>
+      <c r="E197" s="6"/>
+      <c r="F197" s="6"/>
+      <c r="G197" s="6"/>
       <c r="H197" s="2"/>
     </row>
     <row r="198">
       <c r="A198" s="2"/>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C198" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Madison &amp; the War of 1812</t>
-        </is>
-      </c>
-      <c r="D198" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C198" s="5"/>
+      <c r="D198" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Causes and Symbols of the War of 1812</t>
+        </is>
+      </c>
       <c r="E198" s="6"/>
-      <c r="F198" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.5.1, 8.5.2, 8.5.3, 8.12.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
+      <c r="F198" s="6"/>
       <c r="G198" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Why did the United States go to war with Britain in 1812, and how did the war change Americans' sense of national identity?</t>
+          <t xml:space="preserve">6 check questions</t>
         </is>
       </c>
       <c r="H198" s="2"/>
@@ -4154,7 +4154,7 @@
       <c r="C199" s="5"/>
       <c r="D199" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E199" s="6"/>
@@ -4172,7 +4172,7 @@
       <c r="C200" s="5"/>
       <c r="D200" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Madison and the War of 1812</t>
+          <t xml:space="preserve">Interactive Map: Indian Lands Lost by 1810</t>
         </is>
       </c>
       <c r="E200" s="6"/>
@@ -4184,53 +4184,53 @@
       <c r="A201" s="2"/>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C201" s="5"/>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Causes and Symbols of the War of 1812</t>
+          <t xml:space="preserve">Interactive Map: The War of 1812</t>
         </is>
       </c>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
-      <c r="G201" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G201" s="6"/>
       <c r="H201" s="2"/>
     </row>
     <row r="202">
       <c r="A202" s="2"/>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C202" s="5"/>
-      <c r="D202" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D202" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E202" s="6"/>
       <c r="F202" s="6"/>
-      <c r="G202" s="6"/>
+      <c r="G202" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H202" s="2"/>
     </row>
     <row r="203">
       <c r="A203" s="2"/>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C203" s="5"/>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Indian Lands Lost by 1810</t>
+          <t xml:space="preserve">Stranger Than Fiction: The Battle After the Treaty</t>
         </is>
       </c>
       <c r="E203" s="6"/>
@@ -4242,13 +4242,13 @@
       <c r="A204" s="2"/>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C204" s="5"/>
-      <c r="D204" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Map: The War of 1812</t>
+      <c r="D204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E204" s="6"/>
@@ -4266,14 +4266,14 @@
       <c r="C205" s="5"/>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Madison &amp; the War of 1812</t>
         </is>
       </c>
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
       <c r="G205" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H205" s="2"/>
@@ -4282,15 +4282,15 @@
       <c r="A206" s="2"/>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C206" s="5"/>
-      <c r="D206" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Battle After the Treaty</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C206" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Madison &amp; the War of 1812</t>
+        </is>
+      </c>
+      <c r="D206" s="5"/>
       <c r="E206" s="6"/>
       <c r="F206" s="6"/>
       <c r="G206" s="6"/>
@@ -4298,42 +4298,30 @@
     </row>
     <row r="207">
       <c r="A207" s="2"/>
-      <c r="B207" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C207" s="5"/>
-      <c r="D207" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E207" s="6"/>
-      <c r="F207" s="6"/>
-      <c r="G207" s="6"/>
+      <c r="B207" s="2"/>
+      <c r="C207" s="2"/>
+      <c r="D207" s="2"/>
+      <c r="E207" s="2"/>
+      <c r="F207" s="2"/>
+      <c r="G207" s="2"/>
       <c r="H207" s="2"/>
     </row>
     <row r="208">
       <c r="A208" s="2"/>
-      <c r="B208" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C208" s="5"/>
-      <c r="D208" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Madison &amp; the War of 1812</t>
-        </is>
-      </c>
-      <c r="E208" s="6"/>
-      <c r="F208" s="6"/>
-      <c r="G208" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 14</t>
+        </is>
+      </c>
+      <c r="C208" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
+      <c r="D208" s="16"/>
+      <c r="E208" s="16"/>
+      <c r="F208" s="16"/>
+      <c r="G208" s="17"/>
       <c r="H208" s="2"/>
     </row>
     <row r="209">
@@ -4345,65 +4333,77 @@
       </c>
       <c r="C209" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Madison &amp; the War of 1812</t>
+          <t xml:space="preserve">Overview | Monroe's Presidency and Everyday Life</t>
         </is>
       </c>
       <c r="D209" s="5"/>
       <c r="E209" s="6"/>
-      <c r="F209" s="6"/>
-      <c r="G209" s="6"/>
+      <c r="F209" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.3.3, 8.4.1, 8.4.3, 8.4.4, 8.5.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G209" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did the United States grow stronger, more connected, and more divided during Monroe's presidency and the early 1800s?</t>
+        </is>
+      </c>
       <c r="H209" s="2"/>
     </row>
     <row r="210">
       <c r="A210" s="2"/>
-      <c r="B210" s="2"/>
-      <c r="C210" s="2"/>
-      <c r="D210" s="2"/>
-      <c r="E210" s="2"/>
-      <c r="F210" s="2"/>
-      <c r="G210" s="2"/>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C210" s="5"/>
+      <c r="D210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E210" s="6"/>
+      <c r="F210" s="6"/>
+      <c r="G210" s="6"/>
       <c r="H210" s="2"/>
     </row>
     <row r="211">
       <c r="A211" s="2"/>
-      <c r="B211" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 14</t>
-        </is>
-      </c>
-      <c r="C211" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Monroe's Presidency and Everyday Life</t>
-        </is>
-      </c>
-      <c r="D211" s="16"/>
-      <c r="E211" s="16"/>
-      <c r="F211" s="16"/>
-      <c r="G211" s="17"/>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C211" s="5"/>
+      <c r="D211" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
+      <c r="E211" s="6"/>
+      <c r="F211" s="6"/>
+      <c r="G211" s="6"/>
       <c r="H211" s="2"/>
     </row>
     <row r="212">
       <c r="A212" s="2"/>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C212" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Monroe's Presidency and Everyday Life</t>
-        </is>
-      </c>
-      <c r="D212" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C212" s="5"/>
+      <c r="D212" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: The Erie Canal and National Growth</t>
+        </is>
+      </c>
       <c r="E212" s="6"/>
-      <c r="F212" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.3.3, 8.4.1, 8.4.3, 8.4.4, 8.5.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
+      <c r="F212" s="6"/>
       <c r="G212" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">How did the United States grow stronger, more connected, and more divided during Monroe's presidency and the early 1800s?</t>
+          <t xml:space="preserve">6 check questions</t>
         </is>
       </c>
       <c r="H212" s="2"/>
@@ -4418,7 +4418,7 @@
       <c r="C213" s="5"/>
       <c r="D213" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E213" s="6"/>
@@ -4436,7 +4436,7 @@
       <c r="C214" s="5"/>
       <c r="D214" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Monroe's Presidency and Everyday Life</t>
+          <t xml:space="preserve">Interactive Chart: The Beginnings of Sectionalism</t>
         </is>
       </c>
       <c r="E214" s="6"/>
@@ -4448,53 +4448,53 @@
       <c r="A215" s="2"/>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C215" s="5"/>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: The Erie Canal and National Growth</t>
+          <t xml:space="preserve">Interactive Gallery: The Expansion of Federal Power</t>
         </is>
       </c>
       <c r="E215" s="6"/>
       <c r="F215" s="6"/>
-      <c r="G215" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G215" s="6"/>
       <c r="H215" s="2"/>
     </row>
     <row r="216">
       <c r="A216" s="2"/>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C216" s="5"/>
-      <c r="D216" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D216" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E216" s="6"/>
       <c r="F216" s="6"/>
-      <c r="G216" s="6"/>
+      <c r="G216" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H216" s="2"/>
     </row>
     <row r="217">
       <c r="A217" s="2"/>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C217" s="5"/>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: The Beginnings of Sectionalism</t>
+          <t xml:space="preserve">Stranger Than Fiction: The Canal Wedding That Changed America</t>
         </is>
       </c>
       <c r="E217" s="6"/>
@@ -4506,13 +4506,13 @@
       <c r="A218" s="2"/>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C218" s="5"/>
-      <c r="D218" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Gallery: The Expansion of Federal Power</t>
+      <c r="D218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E218" s="6"/>
@@ -4530,14 +4530,14 @@
       <c r="C219" s="5"/>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Monroe's Presidency and Everyday Life</t>
         </is>
       </c>
       <c r="E219" s="6"/>
       <c r="F219" s="6"/>
       <c r="G219" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H219" s="2"/>
@@ -4546,15 +4546,15 @@
       <c r="A220" s="2"/>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C220" s="5"/>
-      <c r="D220" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Canal Wedding That Changed America</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C220" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Monroe's Presidency and Everyday Life</t>
+        </is>
+      </c>
+      <c r="D220" s="5"/>
       <c r="E220" s="6"/>
       <c r="F220" s="6"/>
       <c r="G220" s="6"/>
@@ -4562,42 +4562,30 @@
     </row>
     <row r="221">
       <c r="A221" s="2"/>
-      <c r="B221" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C221" s="5"/>
-      <c r="D221" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E221" s="6"/>
-      <c r="F221" s="6"/>
-      <c r="G221" s="6"/>
+      <c r="B221" s="2"/>
+      <c r="C221" s="2"/>
+      <c r="D221" s="2"/>
+      <c r="E221" s="2"/>
+      <c r="F221" s="2"/>
+      <c r="G221" s="2"/>
       <c r="H221" s="2"/>
     </row>
     <row r="222">
       <c r="A222" s="2"/>
-      <c r="B222" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C222" s="5"/>
-      <c r="D222" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Monroe's Presidency and Everyday Life</t>
-        </is>
-      </c>
-      <c r="E222" s="6"/>
-      <c r="F222" s="6"/>
-      <c r="G222" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 15</t>
+        </is>
+      </c>
+      <c r="C222" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Age of Jackson</t>
+        </is>
+      </c>
+      <c r="D222" s="16"/>
+      <c r="E222" s="16"/>
+      <c r="F222" s="16"/>
+      <c r="G222" s="17"/>
       <c r="H222" s="2"/>
     </row>
     <row r="223">
@@ -4609,98 +4597,110 @@
       </c>
       <c r="C223" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Monroe's Presidency and Everyday Life</t>
+          <t xml:space="preserve">Overview | The Age of Jackson</t>
         </is>
       </c>
       <c r="D223" s="5"/>
       <c r="E223" s="6"/>
-      <c r="F223" s="6"/>
-      <c r="G223" s="6"/>
+      <c r="F223" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.6.6, 8.8.1, 8.10.2, 8.4.3, 8.9.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G223" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Andrew Jackson's presidency expand democracy for some Americans while increasing conflict over power, money, and rights?</t>
+        </is>
+      </c>
       <c r="H223" s="2"/>
     </row>
     <row r="224">
       <c r="A224" s="2"/>
-      <c r="B224" s="2"/>
-      <c r="C224" s="2"/>
-      <c r="D224" s="2"/>
-      <c r="E224" s="2"/>
-      <c r="F224" s="2"/>
-      <c r="G224" s="2"/>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C224" s="5"/>
+      <c r="D224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E224" s="6"/>
+      <c r="F224" s="6"/>
+      <c r="G224" s="6"/>
       <c r="H224" s="2"/>
     </row>
     <row r="225">
       <c r="A225" s="2"/>
-      <c r="B225" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 15</t>
-        </is>
-      </c>
-      <c r="C225" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Age of Jackson</t>
-        </is>
-      </c>
-      <c r="D225" s="16"/>
-      <c r="E225" s="16"/>
-      <c r="F225" s="16"/>
-      <c r="G225" s="17"/>
+      <c r="B225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C225" s="5"/>
+      <c r="D225" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Jackson Wins the Presidency</t>
+        </is>
+      </c>
+      <c r="E225" s="6"/>
+      <c r="F225" s="6"/>
+      <c r="G225" s="6"/>
       <c r="H225" s="2"/>
     </row>
     <row r="226">
       <c r="A226" s="2"/>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C226" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The Age of Jackson</t>
-        </is>
-      </c>
-      <c r="D226" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C226" s="5"/>
+      <c r="D226" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Political Conflict and Economic Crisis</t>
+        </is>
+      </c>
       <c r="E226" s="6"/>
-      <c r="F226" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.6.6, 8.8.1, 8.10.2, 8.4.3, 8.9.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G226" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did Andrew Jackson's presidency expand democracy for some Americans while increasing conflict over power, money, and rights?</t>
-        </is>
-      </c>
+      <c r="F226" s="6"/>
+      <c r="G226" s="6"/>
       <c r="H226" s="2"/>
     </row>
     <row r="227">
       <c r="A227" s="2"/>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C227" s="5"/>
-      <c r="D227" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D227" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Andrew Jackson and the Age of Jackson</t>
         </is>
       </c>
       <c r="E227" s="6"/>
       <c r="F227" s="6"/>
-      <c r="G227" s="6"/>
+      <c r="G227" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H227" s="2"/>
     </row>
     <row r="228">
       <c r="A228" s="2"/>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C228" s="5"/>
-      <c r="D228" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Jackson Wins the Presidency</t>
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E228" s="6"/>
@@ -4718,7 +4718,7 @@
       <c r="C229" s="5"/>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Political Conflict and Economic Crisis</t>
+          <t xml:space="preserve">Interactive Timeline: Changing Voting Rights in Early America</t>
         </is>
       </c>
       <c r="E229" s="6"/>
@@ -4730,35 +4730,31 @@
       <c r="A230" s="2"/>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C230" s="5"/>
       <c r="D230" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Andrew Jackson and the Age of Jackson</t>
+          <t xml:space="preserve">Interactive Chart: Political Parties in the Age of Jackson</t>
         </is>
       </c>
       <c r="E230" s="6"/>
       <c r="F230" s="6"/>
-      <c r="G230" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G230" s="6"/>
       <c r="H230" s="2"/>
     </row>
     <row r="231">
       <c r="A231" s="2"/>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C231" s="5"/>
-      <c r="D231" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D231" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Tariffs and Trade</t>
         </is>
       </c>
       <c r="E231" s="6"/>
@@ -4776,7 +4772,7 @@
       <c r="C232" s="5"/>
       <c r="D232" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Timeline: Changing Voting Rights in Early America</t>
+          <t xml:space="preserve">Interactive Chart: Disagreements Over the Bank</t>
         </is>
       </c>
       <c r="E232" s="6"/>
@@ -4788,49 +4784,57 @@
       <c r="A233" s="2"/>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C233" s="5"/>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Chart: Political Parties in the Age of Jackson</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E233" s="6"/>
       <c r="F233" s="6"/>
-      <c r="G233" s="6"/>
+      <c r="G233" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H233" s="2"/>
     </row>
     <row r="234">
       <c r="A234" s="2"/>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C234" s="5"/>
       <c r="D234" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Tariffs and Trade</t>
+          <t xml:space="preserve">Stranger Than Fiction: Old Hickory Would Not Back Down</t>
         </is>
       </c>
       <c r="E234" s="6"/>
       <c r="F234" s="6"/>
-      <c r="G234" s="6"/>
+      <c r="G234" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drag-and-drop</t>
+        </is>
+      </c>
       <c r="H234" s="2"/>
     </row>
     <row r="235">
       <c r="A235" s="2"/>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C235" s="5"/>
-      <c r="D235" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Chart: Disagreements Over the Bank</t>
+      <c r="D235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E235" s="6"/>
@@ -4848,14 +4852,14 @@
       <c r="C236" s="5"/>
       <c r="D236" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: The Age of Jackson</t>
         </is>
       </c>
       <c r="E236" s="6"/>
       <c r="F236" s="6"/>
       <c r="G236" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H236" s="2"/>
@@ -4864,62 +4868,46 @@
       <c r="A237" s="2"/>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C237" s="5"/>
-      <c r="D237" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: Old Hickory Would Not Back Down</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C237" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Age of Jackson</t>
+        </is>
+      </c>
+      <c r="D237" s="5"/>
       <c r="E237" s="6"/>
       <c r="F237" s="6"/>
-      <c r="G237" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">drag-and-drop</t>
-        </is>
-      </c>
+      <c r="G237" s="6"/>
       <c r="H237" s="2"/>
     </row>
     <row r="238">
       <c r="A238" s="2"/>
-      <c r="B238" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C238" s="5"/>
-      <c r="D238" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E238" s="6"/>
-      <c r="F238" s="6"/>
-      <c r="G238" s="6"/>
+      <c r="B238" s="2"/>
+      <c r="C238" s="2"/>
+      <c r="D238" s="2"/>
+      <c r="E238" s="2"/>
+      <c r="F238" s="2"/>
+      <c r="G238" s="2"/>
       <c r="H238" s="2"/>
     </row>
     <row r="239">
       <c r="A239" s="2"/>
-      <c r="B239" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C239" s="5"/>
-      <c r="D239" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: The Age of Jackson</t>
-        </is>
-      </c>
-      <c r="E239" s="6"/>
-      <c r="F239" s="6"/>
-      <c r="G239" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 16</t>
+        </is>
+      </c>
+      <c r="C239" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">American Indians &amp; Westward Movement</t>
+        </is>
+      </c>
+      <c r="D239" s="16"/>
+      <c r="E239" s="16"/>
+      <c r="F239" s="16"/>
+      <c r="G239" s="17"/>
       <c r="H239" s="2"/>
     </row>
     <row r="240">
@@ -4931,98 +4919,110 @@
       </c>
       <c r="C240" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | The Age of Jackson</t>
+          <t xml:space="preserve">Overview | American Indians &amp; Westward Movement</t>
         </is>
       </c>
       <c r="D240" s="5"/>
       <c r="E240" s="6"/>
-      <c r="F240" s="6"/>
-      <c r="G240" s="6"/>
+      <c r="F240" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.8.1, 8.8.2, 8.12.2, 8.6.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G240" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did westward expansion affect American Indian nations and settlers, and what happens when law on paper does not match power in practice?</t>
+        </is>
+      </c>
       <c r="H240" s="2"/>
     </row>
     <row r="241">
       <c r="A241" s="2"/>
-      <c r="B241" s="2"/>
-      <c r="C241" s="2"/>
-      <c r="D241" s="2"/>
-      <c r="E241" s="2"/>
-      <c r="F241" s="2"/>
-      <c r="G241" s="2"/>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C241" s="5"/>
+      <c r="D241" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E241" s="6"/>
+      <c r="F241" s="6"/>
+      <c r="G241" s="6"/>
       <c r="H241" s="2"/>
     </row>
     <row r="242">
       <c r="A242" s="2"/>
-      <c r="B242" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 16</t>
-        </is>
-      </c>
-      <c r="C242" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">American Indians &amp; Westward Movement</t>
-        </is>
-      </c>
-      <c r="D242" s="16"/>
-      <c r="E242" s="16"/>
-      <c r="F242" s="16"/>
-      <c r="G242" s="17"/>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C242" s="5"/>
+      <c r="D242" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Conflict with American Indians</t>
+        </is>
+      </c>
+      <c r="E242" s="6"/>
+      <c r="F242" s="6"/>
+      <c r="G242" s="6"/>
       <c r="H242" s="2"/>
     </row>
     <row r="243">
       <c r="A243" s="2"/>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C243" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | American Indians &amp; Westward Movement</t>
-        </is>
-      </c>
-      <c r="D243" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C243" s="5"/>
+      <c r="D243" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Westward Movement</t>
+        </is>
+      </c>
       <c r="E243" s="6"/>
-      <c r="F243" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.8.1, 8.8.2, 8.12.2, 8.6.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G243" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How did westward expansion affect American Indian nations and settlers, and what happens when law on paper does not match power in practice?</t>
-        </is>
-      </c>
+      <c r="F243" s="6"/>
+      <c r="G243" s="6"/>
       <c r="H243" s="2"/>
     </row>
     <row r="244">
       <c r="A244" s="2"/>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C244" s="5"/>
-      <c r="D244" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D244" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Removal, Law, and Westward Movement</t>
         </is>
       </c>
       <c r="E244" s="6"/>
       <c r="F244" s="6"/>
-      <c r="G244" s="6"/>
+      <c r="G244" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H244" s="2"/>
     </row>
     <row r="245">
       <c r="A245" s="2"/>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C245" s="5"/>
-      <c r="D245" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Conflict with American Indians</t>
+      <c r="D245" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E245" s="6"/>
@@ -5040,7 +5040,7 @@
       <c r="C246" s="5"/>
       <c r="D246" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Westward Movement</t>
+          <t xml:space="preserve">Interactive Map: Selected Native American Groups</t>
         </is>
       </c>
       <c r="E246" s="6"/>
@@ -5052,35 +5052,31 @@
       <c r="A247" s="2"/>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C247" s="5"/>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Removal, Law, and Westward Movement</t>
+          <t xml:space="preserve">Interactive Map: The Trail of Tears</t>
         </is>
       </c>
       <c r="E247" s="6"/>
       <c r="F247" s="6"/>
-      <c r="G247" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G247" s="6"/>
       <c r="H247" s="2"/>
     </row>
     <row r="248">
       <c r="A248" s="2"/>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C248" s="5"/>
-      <c r="D248" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D248" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: New Transportation Methods</t>
         </is>
       </c>
       <c r="E248" s="6"/>
@@ -5098,7 +5094,7 @@
       <c r="C249" s="5"/>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Selected Native American Groups</t>
+          <t xml:space="preserve">Interactive Gallery: New Technology: The Steamboat</t>
         </is>
       </c>
       <c r="E249" s="6"/>
@@ -5110,49 +5106,57 @@
       <c r="A250" s="2"/>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C250" s="5"/>
       <c r="D250" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: The Trail of Tears</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E250" s="6"/>
       <c r="F250" s="6"/>
-      <c r="G250" s="6"/>
+      <c r="G250" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H250" s="2"/>
     </row>
     <row r="251">
       <c r="A251" s="2"/>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C251" s="5"/>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: New Transportation Methods</t>
+          <t xml:space="preserve">Stranger Than Fiction: The Cherokee Won, Then Lost It All</t>
         </is>
       </c>
       <c r="E251" s="6"/>
       <c r="F251" s="6"/>
-      <c r="G251" s="6"/>
+      <c r="G251" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">drag-and-drop</t>
+        </is>
+      </c>
       <c r="H251" s="2"/>
     </row>
     <row r="252">
       <c r="A252" s="2"/>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C252" s="5"/>
-      <c r="D252" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Gallery: New Technology: The Steamboat</t>
+      <c r="D252" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E252" s="6"/>
@@ -5170,14 +5174,14 @@
       <c r="C253" s="5"/>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: American Indians &amp; Westward Movement</t>
         </is>
       </c>
       <c r="E253" s="6"/>
       <c r="F253" s="6"/>
       <c r="G253" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H253" s="2"/>
@@ -5186,62 +5190,46 @@
       <c r="A254" s="2"/>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C254" s="5"/>
-      <c r="D254" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Cherokee Won, Then Lost It All</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C254" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | American Indians &amp; Westward Movement</t>
+        </is>
+      </c>
+      <c r="D254" s="5"/>
       <c r="E254" s="6"/>
       <c r="F254" s="6"/>
-      <c r="G254" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">drag-and-drop</t>
-        </is>
-      </c>
+      <c r="G254" s="6"/>
       <c r="H254" s="2"/>
     </row>
     <row r="255">
       <c r="A255" s="2"/>
-      <c r="B255" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C255" s="5"/>
-      <c r="D255" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E255" s="6"/>
-      <c r="F255" s="6"/>
-      <c r="G255" s="6"/>
+      <c r="B255" s="2"/>
+      <c r="C255" s="2"/>
+      <c r="D255" s="2"/>
+      <c r="E255" s="2"/>
+      <c r="F255" s="2"/>
+      <c r="G255" s="2"/>
       <c r="H255" s="2"/>
     </row>
     <row r="256">
       <c r="A256" s="2"/>
-      <c r="B256" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C256" s="5"/>
-      <c r="D256" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: American Indians &amp; Westward Movement</t>
-        </is>
-      </c>
-      <c r="E256" s="6"/>
-      <c r="F256" s="6"/>
-      <c r="G256" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 17</t>
+        </is>
+      </c>
+      <c r="C256" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Settling Oregon &amp; Independence for Texas</t>
+        </is>
+      </c>
+      <c r="D256" s="16"/>
+      <c r="E256" s="16"/>
+      <c r="F256" s="16"/>
+      <c r="G256" s="17"/>
       <c r="H256" s="2"/>
     </row>
     <row r="257">
@@ -5253,98 +5241,110 @@
       </c>
       <c r="C257" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | American Indians &amp; Westward Movement</t>
+          <t xml:space="preserve">Overview | Settling Oregon &amp; Independence for Texas</t>
         </is>
       </c>
       <c r="D257" s="5"/>
       <c r="E257" s="6"/>
-      <c r="F257" s="6"/>
-      <c r="G257" s="6"/>
+      <c r="F257" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.8.2, 8.8.3, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G257" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why did Americans move into Oregon and Texas, and how did settlement in the West create new conflicts over land, independence, and annexation?</t>
+        </is>
+      </c>
       <c r="H257" s="2"/>
     </row>
     <row r="258">
       <c r="A258" s="2"/>
-      <c r="B258" s="2"/>
-      <c r="C258" s="2"/>
-      <c r="D258" s="2"/>
-      <c r="E258" s="2"/>
-      <c r="F258" s="2"/>
-      <c r="G258" s="2"/>
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C258" s="5"/>
+      <c r="D258" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E258" s="6"/>
+      <c r="F258" s="6"/>
+      <c r="G258" s="6"/>
       <c r="H258" s="2"/>
     </row>
     <row r="259">
       <c r="A259" s="2"/>
-      <c r="B259" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 17</t>
-        </is>
-      </c>
-      <c r="C259" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Settling Oregon &amp; Independence for Texas</t>
-        </is>
-      </c>
-      <c r="D259" s="16"/>
-      <c r="E259" s="16"/>
-      <c r="F259" s="16"/>
-      <c r="G259" s="17"/>
+      <c r="B259" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C259" s="5"/>
+      <c r="D259" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Settling Oregon Country</t>
+        </is>
+      </c>
+      <c r="E259" s="6"/>
+      <c r="F259" s="6"/>
+      <c r="G259" s="6"/>
       <c r="H259" s="2"/>
     </row>
     <row r="260">
       <c r="A260" s="2"/>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C260" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Settling Oregon &amp; Independence for Texas</t>
-        </is>
-      </c>
-      <c r="D260" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C260" s="5"/>
+      <c r="D260" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: New Spain and Independence for Texas</t>
+        </is>
+      </c>
       <c r="E260" s="6"/>
-      <c r="F260" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.8.2, 8.8.3, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
-      <c r="G260" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Why did Americans move into Oregon and Texas, and how did settlement in the West create new conflicts over land, independence, and annexation?</t>
-        </is>
-      </c>
+      <c r="F260" s="6"/>
+      <c r="G260" s="6"/>
       <c r="H260" s="2"/>
     </row>
     <row r="261">
       <c r="A261" s="2"/>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C261" s="5"/>
-      <c r="D261" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D261" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Oregon, Texas, and Westward Settlement</t>
         </is>
       </c>
       <c r="E261" s="6"/>
       <c r="F261" s="6"/>
-      <c r="G261" s="6"/>
+      <c r="G261" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H261" s="2"/>
     </row>
     <row r="262">
       <c r="A262" s="2"/>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C262" s="5"/>
-      <c r="D262" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eText: Settling Oregon Country</t>
+      <c r="D262" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E262" s="6"/>
@@ -5362,7 +5362,7 @@
       <c r="C263" s="5"/>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: New Spain and Independence for Texas</t>
+          <t xml:space="preserve">Interactive Map: Trails West</t>
         </is>
       </c>
       <c r="E263" s="6"/>
@@ -5374,35 +5374,31 @@
       <c r="A264" s="2"/>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C264" s="5"/>
       <c r="D264" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Oregon, Texas, and Westward Settlement</t>
+          <t xml:space="preserve">Interactive Gallery: Life on the Oregon Trail</t>
         </is>
       </c>
       <c r="E264" s="6"/>
       <c r="F264" s="6"/>
-      <c r="G264" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G264" s="6"/>
       <c r="H264" s="2"/>
     </row>
     <row r="265">
       <c r="A265" s="2"/>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C265" s="5"/>
-      <c r="D265" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D265" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Texas and the Southwest</t>
         </is>
       </c>
       <c r="E265" s="6"/>
@@ -5420,7 +5416,7 @@
       <c r="C266" s="5"/>
       <c r="D266" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Trails West</t>
+          <t xml:space="preserve">Interactive Timeline: Independence for Texas</t>
         </is>
       </c>
       <c r="E266" s="6"/>
@@ -5432,31 +5428,35 @@
       <c r="A267" s="2"/>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C267" s="5"/>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Gallery: Life on the Oregon Trail</t>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E267" s="6"/>
       <c r="F267" s="6"/>
-      <c r="G267" s="6"/>
+      <c r="G267" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H267" s="2"/>
     </row>
     <row r="268">
       <c r="A268" s="2"/>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C268" s="5"/>
       <c r="D268" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: Texas and the Southwest</t>
+          <t xml:space="preserve">Stranger Than Fiction: Texas Was Its Own Country</t>
         </is>
       </c>
       <c r="E268" s="6"/>
@@ -5468,13 +5468,13 @@
       <c r="A269" s="2"/>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C269" s="5"/>
-      <c r="D269" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Timeline: Independence for Texas</t>
+      <c r="D269" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E269" s="6"/>
@@ -5492,14 +5492,14 @@
       <c r="C270" s="5"/>
       <c r="D270" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Settling Oregon &amp; Independence for Texas</t>
         </is>
       </c>
       <c r="E270" s="6"/>
       <c r="F270" s="6"/>
       <c r="G270" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H270" s="2"/>
@@ -5508,15 +5508,15 @@
       <c r="A271" s="2"/>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C271" s="5"/>
-      <c r="D271" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: Texas Was Its Own Country</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C271" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Settling Oregon &amp; Independence for Texas</t>
+        </is>
+      </c>
+      <c r="D271" s="5"/>
       <c r="E271" s="6"/>
       <c r="F271" s="6"/>
       <c r="G271" s="6"/>
@@ -5524,42 +5524,30 @@
     </row>
     <row r="272">
       <c r="A272" s="2"/>
-      <c r="B272" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C272" s="5"/>
-      <c r="D272" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E272" s="6"/>
-      <c r="F272" s="6"/>
-      <c r="G272" s="6"/>
+      <c r="B272" s="2"/>
+      <c r="C272" s="2"/>
+      <c r="D272" s="2"/>
+      <c r="E272" s="2"/>
+      <c r="F272" s="2"/>
+      <c r="G272" s="2"/>
       <c r="H272" s="2"/>
     </row>
     <row r="273">
       <c r="A273" s="2"/>
-      <c r="B273" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C273" s="5"/>
-      <c r="D273" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Settling Oregon &amp; Independence for Texas</t>
-        </is>
-      </c>
-      <c r="E273" s="6"/>
-      <c r="F273" s="6"/>
-      <c r="G273" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 18</t>
+        </is>
+      </c>
+      <c r="C273" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manifest Destiny in California &amp; the Southwest</t>
+        </is>
+      </c>
+      <c r="D273" s="16"/>
+      <c r="E273" s="16"/>
+      <c r="F273" s="16"/>
+      <c r="G273" s="17"/>
       <c r="H273" s="2"/>
     </row>
     <row r="274">
@@ -5571,65 +5559,77 @@
       </c>
       <c r="C274" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Settling Oregon &amp; Independence for Texas</t>
+          <t xml:space="preserve">Overview | Manifest Destiny in California &amp; the Southwest</t>
         </is>
       </c>
       <c r="D274" s="5"/>
       <c r="E274" s="6"/>
-      <c r="F274" s="6"/>
-      <c r="G274" s="6"/>
+      <c r="F274" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.5.2, 8.6.2, 8.8.1, 8.8.2, 8.8.4, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G274" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Manifest Destiny and the Mexican-American War change California, the Southwest, and the United States?</t>
+        </is>
+      </c>
       <c r="H274" s="2"/>
     </row>
     <row r="275">
       <c r="A275" s="2"/>
-      <c r="B275" s="2"/>
-      <c r="C275" s="2"/>
-      <c r="D275" s="2"/>
-      <c r="E275" s="2"/>
-      <c r="F275" s="2"/>
-      <c r="G275" s="2"/>
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C275" s="5"/>
+      <c r="D275" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E275" s="6"/>
+      <c r="F275" s="6"/>
+      <c r="G275" s="6"/>
       <c r="H275" s="2"/>
     </row>
     <row r="276">
       <c r="A276" s="2"/>
-      <c r="B276" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 18</t>
-        </is>
-      </c>
-      <c r="C276" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manifest Destiny in California &amp; the Southwest</t>
-        </is>
-      </c>
-      <c r="D276" s="16"/>
-      <c r="E276" s="16"/>
-      <c r="F276" s="16"/>
-      <c r="G276" s="17"/>
+      <c r="B276" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C276" s="5"/>
+      <c r="D276" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Manifest Destiny in California and the Southwest</t>
+        </is>
+      </c>
+      <c r="E276" s="6"/>
+      <c r="F276" s="6"/>
+      <c r="G276" s="6"/>
       <c r="H276" s="2"/>
     </row>
     <row r="277">
       <c r="A277" s="2"/>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C277" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Manifest Destiny in California &amp; the Southwest</t>
-        </is>
-      </c>
-      <c r="D277" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C277" s="5"/>
+      <c r="D277" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Manifest Destiny and the Mexican-American War</t>
+        </is>
+      </c>
       <c r="E277" s="6"/>
-      <c r="F277" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.5.2, 8.6.2, 8.8.1, 8.8.2, 8.8.4, 8.8.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.7, RI.8.8 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
-        </is>
-      </c>
+      <c r="F277" s="6"/>
       <c r="G277" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">How did Manifest Destiny and the Mexican-American War change California, the Southwest, and the United States?</t>
+          <t xml:space="preserve">6 check questions</t>
         </is>
       </c>
       <c r="H277" s="2"/>
@@ -5644,7 +5644,7 @@
       <c r="C278" s="5"/>
       <c r="D278" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E278" s="6"/>
@@ -5662,7 +5662,7 @@
       <c r="C279" s="5"/>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">eText: Manifest Destiny in California and the Southwest</t>
+          <t xml:space="preserve">Interactive Map: The Growth of the West to 1860</t>
         </is>
       </c>
       <c r="E279" s="6"/>
@@ -5674,53 +5674,53 @@
       <c r="A280" s="2"/>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Assignment</t>
         </is>
       </c>
       <c r="C280" s="5"/>
       <c r="D280" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Video: Manifest Destiny and the Mexican-American War</t>
+          <t xml:space="preserve">Interactive Gallery: The People of California</t>
         </is>
       </c>
       <c r="E280" s="6"/>
       <c r="F280" s="6"/>
-      <c r="G280" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 check questions</t>
-        </is>
-      </c>
+      <c r="G280" s="6"/>
       <c r="H280" s="2"/>
     </row>
     <row r="281">
       <c r="A281" s="2"/>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C281" s="5"/>
-      <c r="D281" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D281" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E281" s="6"/>
       <c r="F281" s="6"/>
-      <c r="G281" s="6"/>
+      <c r="G281" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H281" s="2"/>
     </row>
     <row r="282">
       <c r="A282" s="2"/>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="C282" s="5"/>
       <c r="D282" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Map: The Growth of the West to 1860</t>
+          <t xml:space="preserve">Stranger Than Fiction: The Bear Flag Republic: It Bearly Lasted a Month</t>
         </is>
       </c>
       <c r="E282" s="6"/>
@@ -5732,13 +5732,13 @@
       <c r="A283" s="2"/>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assignment</t>
+          <t xml:space="preserve">Text Header</t>
         </is>
       </c>
       <c r="C283" s="5"/>
-      <c r="D283" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interactive Gallery: The People of California</t>
+      <c r="D283" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E283" s="6"/>
@@ -5756,14 +5756,14 @@
       <c r="C284" s="5"/>
       <c r="D284" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check for Understanding</t>
+          <t xml:space="preserve">Module Quiz: Manifest Destiny in California &amp; the Southwest</t>
         </is>
       </c>
       <c r="E284" s="6"/>
       <c r="F284" s="6"/>
       <c r="G284" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 questions</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H284" s="2"/>
@@ -5772,15 +5772,15 @@
       <c r="A285" s="2"/>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C285" s="5"/>
-      <c r="D285" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stranger Than Fiction: The Bear Flag Republic: It Bearly Lasted a Month</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C285" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Manifest Destiny in California &amp; the Southwest</t>
+        </is>
+      </c>
+      <c r="D285" s="5"/>
       <c r="E285" s="6"/>
       <c r="F285" s="6"/>
       <c r="G285" s="6"/>
@@ -5788,42 +5788,30 @@
     </row>
     <row r="286">
       <c r="A286" s="2"/>
-      <c r="B286" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C286" s="5"/>
-      <c r="D286" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E286" s="6"/>
-      <c r="F286" s="6"/>
-      <c r="G286" s="6"/>
+      <c r="B286" s="2"/>
+      <c r="C286" s="2"/>
+      <c r="D286" s="2"/>
+      <c r="E286" s="2"/>
+      <c r="F286" s="2"/>
+      <c r="G286" s="2"/>
       <c r="H286" s="2"/>
     </row>
     <row r="287">
       <c r="A287" s="2"/>
-      <c r="B287" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="C287" s="5"/>
-      <c r="D287" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Module Quiz: Manifest Destiny in California &amp; the Southwest</t>
-        </is>
-      </c>
-      <c r="E287" s="6"/>
-      <c r="F287" s="6"/>
-      <c r="G287" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pool 15, draws 10</t>
-        </is>
-      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 19</t>
+        </is>
+      </c>
+      <c r="C287" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Current Events Connection  (Project)</t>
+        </is>
+      </c>
+      <c r="D287" s="16"/>
+      <c r="E287" s="16"/>
+      <c r="F287" s="16"/>
+      <c r="G287" s="17"/>
       <c r="H287" s="2"/>
     </row>
     <row r="288">
@@ -5835,82 +5823,90 @@
       </c>
       <c r="C288" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Manifest Destiny in California &amp; the Southwest</t>
+          <t xml:space="preserve">Overview | PROJECT - Current Events Connection</t>
         </is>
       </c>
       <c r="D288" s="5"/>
       <c r="E288" s="6"/>
-      <c r="F288" s="6"/>
-      <c r="G288" s="6"/>
+      <c r="F288" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS Course-specific social science content standards connected to the student's chosen topic | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.7, W.8.8, W.8.9, SL.8.4, SL.8.5 | ELD Part I A.3, Part I B.6, Part I B.7, Part I C.10, Part I C.11</t>
+        </is>
+      </c>
+      <c r="G288" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How can a current event help us understand patterns, conflicts, and choices from the past?</t>
+        </is>
+      </c>
       <c r="H288" s="2"/>
     </row>
     <row r="289">
       <c r="A289" s="2"/>
-      <c r="B289" s="2"/>
-      <c r="C289" s="2"/>
-      <c r="D289" s="2"/>
-      <c r="E289" s="2"/>
-      <c r="F289" s="2"/>
-      <c r="G289" s="2"/>
+      <c r="B289" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C289" s="5"/>
+      <c r="D289" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E289" s="6"/>
+      <c r="F289" s="6"/>
+      <c r="G289" s="6"/>
       <c r="H289" s="2"/>
     </row>
     <row r="290">
       <c r="A290" s="2"/>
-      <c r="B290" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 19</t>
-        </is>
-      </c>
-      <c r="C290" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT - Current Events Connection  (Project)</t>
-        </is>
-      </c>
-      <c r="D290" s="16"/>
-      <c r="E290" s="16"/>
-      <c r="F290" s="16"/>
-      <c r="G290" s="17"/>
+      <c r="B290" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C290" s="5"/>
+      <c r="D290" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E290" s="6"/>
+      <c r="F290" s="6"/>
+      <c r="G290" s="6"/>
       <c r="H290" s="2"/>
     </row>
     <row r="291">
       <c r="A291" s="2"/>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C291" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT - Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D291" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C291" s="5"/>
+      <c r="D291" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E291" s="6"/>
-      <c r="F291" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS Course-specific social science content standards connected to the student's chosen topic | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.7, W.8.8, W.8.9, SL.8.4, SL.8.5 | ELD Part I A.3, Part I B.6, Part I B.7, Part I C.10, Part I C.11</t>
-        </is>
-      </c>
-      <c r="G291" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How can a current event help us understand patterns, conflicts, and choices from the past?</t>
-        </is>
-      </c>
+      <c r="F291" s="6"/>
+      <c r="G291" s="6"/>
       <c r="H291" s="2"/>
     </row>
     <row r="292">
       <c r="A292" s="2"/>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C292" s="5"/>
-      <c r="D292" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C292" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D292" s="5"/>
       <c r="E292" s="6"/>
       <c r="F292" s="6"/>
       <c r="G292" s="6"/>
@@ -5918,38 +5914,30 @@
     </row>
     <row r="293">
       <c r="A293" s="2"/>
-      <c r="B293" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C293" s="5"/>
-      <c r="D293" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E293" s="6"/>
-      <c r="F293" s="6"/>
-      <c r="G293" s="6"/>
+      <c r="B293" s="2"/>
+      <c r="C293" s="2"/>
+      <c r="D293" s="2"/>
+      <c r="E293" s="2"/>
+      <c r="F293" s="2"/>
+      <c r="G293" s="2"/>
       <c r="H293" s="2"/>
     </row>
     <row r="294">
       <c r="A294" s="2"/>
-      <c r="B294" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C294" s="5"/>
-      <c r="D294" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E294" s="6"/>
-      <c r="F294" s="6"/>
-      <c r="G294" s="6"/>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 20</t>
+        </is>
+      </c>
+      <c r="C294" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study Guide &amp; Final Exam  (Exam)</t>
+        </is>
+      </c>
+      <c r="D294" s="16"/>
+      <c r="E294" s="16"/>
+      <c r="F294" s="16"/>
+      <c r="G294" s="17"/>
       <c r="H294" s="2"/>
     </row>
     <row r="295">
@@ -5961,41 +5949,57 @@
       </c>
       <c r="C295" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
+          <t xml:space="preserve">Overview | Study Guide &amp; Final Exam</t>
         </is>
       </c>
       <c r="D295" s="5"/>
       <c r="E295" s="6"/>
       <c r="F295" s="6"/>
-      <c r="G295" s="6"/>
+      <c r="G295" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semester 1 review and final exam</t>
+        </is>
+      </c>
       <c r="H295" s="2"/>
     </row>
     <row r="296">
       <c r="A296" s="2"/>
-      <c r="B296" s="2"/>
-      <c r="C296" s="2"/>
-      <c r="D296" s="2"/>
-      <c r="E296" s="2"/>
-      <c r="F296" s="2"/>
-      <c r="G296" s="2"/>
+      <c r="B296" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C296" s="5"/>
+      <c r="D296" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study Guide and Final Exam</t>
+        </is>
+      </c>
+      <c r="E296" s="6"/>
+      <c r="F296" s="6"/>
+      <c r="G296" s="6"/>
       <c r="H296" s="2"/>
     </row>
     <row r="297">
       <c r="A297" s="2"/>
-      <c r="B297" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 20</t>
-        </is>
-      </c>
-      <c r="C297" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Study Guide &amp; Final Exam  (Exam)</t>
-        </is>
-      </c>
-      <c r="D297" s="16"/>
-      <c r="E297" s="16"/>
-      <c r="F297" s="16"/>
-      <c r="G297" s="17"/>
+      <c r="B297" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C297" s="5"/>
+      <c r="D297" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20.1 | Semester 1 Final Exam Study Guide</t>
+        </is>
+      </c>
+      <c r="E297" s="6"/>
+      <c r="F297" s="6"/>
+      <c r="G297" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Download the study guide, answer the questions in your own words, and study from your answers before the final exam. Download: US History 8-1 Final Exam Study Guide.docx</t>
+        </is>
+      </c>
       <c r="H297" s="2"/>
     </row>
     <row r="298">
@@ -6005,17 +6009,17 @@
           <t xml:space="preserve">Page</t>
         </is>
       </c>
-      <c r="C298" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Study Guide &amp; Final Exam</t>
-        </is>
-      </c>
-      <c r="D298" s="5"/>
+      <c r="C298" s="5"/>
+      <c r="D298" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20.2 | Semester 1 Final Exam (Midterm)</t>
+        </is>
+      </c>
       <c r="E298" s="6"/>
       <c r="F298" s="6"/>
       <c r="G298" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Semester 1 review and final exam</t>
+          <t xml:space="preserve">Your teacher will tell you when and where to complete the Semester 1 Final Exam. This may also be called the midterm.</t>
         </is>
       </c>
       <c r="H298" s="2"/>
@@ -6030,7 +6034,7 @@
       <c r="C299" s="5"/>
       <c r="D299" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Study Guide and Final Exam</t>
+          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
         </is>
       </c>
       <c r="E299" s="6"/>
@@ -6042,20 +6046,20 @@
       <c r="A300" s="2"/>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
+          <t xml:space="preserve">Resource</t>
         </is>
       </c>
       <c r="C300" s="5"/>
       <c r="D300" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">20.1 | Semester 1 Final Exam Study Guide</t>
+          <t xml:space="preserve">Printable study guide Word document</t>
         </is>
       </c>
       <c r="E300" s="6"/>
       <c r="F300" s="6"/>
       <c r="G300" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download the study guide, answer the questions in your own words, and study from your answers before the final exam. Download: US History 8-1 Final Exam Study Guide.docx</t>
+          <t xml:space="preserve">course_planning/content/8-1/module-20-assets/US-History-8-1-Final-Exam-Study-Guide.docx</t>
         </is>
       </c>
       <c r="H300" s="2"/>
@@ -6067,92 +6071,30 @@
           <t xml:space="preserve">Page</t>
         </is>
       </c>
-      <c r="C301" s="5"/>
-      <c r="D301" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20.2 | Semester 1 Final Exam (Midterm)</t>
-        </is>
-      </c>
+      <c r="C301" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D301" s="5"/>
       <c r="E301" s="6"/>
       <c r="F301" s="6"/>
       <c r="G301" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your teacher will tell you when and where to complete the Semester 1 Final Exam. This may also be called the midterm.</t>
+          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module only contains review directions and the downloadable study guide.</t>
         </is>
       </c>
       <c r="H301" s="2"/>
     </row>
     <row r="302">
       <c r="A302" s="2"/>
-      <c r="B302" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C302" s="5"/>
-      <c r="D302" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
-        </is>
-      </c>
-      <c r="E302" s="6"/>
-      <c r="F302" s="6"/>
-      <c r="G302" s="6"/>
+      <c r="B302" s="2"/>
+      <c r="C302" s="2"/>
+      <c r="D302" s="2"/>
+      <c r="E302" s="2"/>
+      <c r="F302" s="2"/>
+      <c r="G302" s="2"/>
       <c r="H302" s="2"/>
-    </row>
-    <row r="303">
-      <c r="A303" s="2"/>
-      <c r="B303" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Resource</t>
-        </is>
-      </c>
-      <c r="C303" s="5"/>
-      <c r="D303" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Printable study guide Word document</t>
-        </is>
-      </c>
-      <c r="E303" s="6"/>
-      <c r="F303" s="6"/>
-      <c r="G303" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">course_planning/content/8-1/module-20-assets/US-History-8-1-Final-Exam-Study-Guide.docx</t>
-        </is>
-      </c>
-      <c r="H303" s="2"/>
-    </row>
-    <row r="304">
-      <c r="A304" s="2"/>
-      <c r="B304" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C304" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
-        </is>
-      </c>
-      <c r="D304" s="5"/>
-      <c r="E304" s="6"/>
-      <c r="F304" s="6"/>
-      <c r="G304" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module only contains review directions and the downloadable study guide.</t>
-        </is>
-      </c>
-      <c r="H304" s="2"/>
-    </row>
-    <row r="305">
-      <c r="A305" s="2"/>
-      <c r="B305" s="2"/>
-      <c r="C305" s="2"/>
-      <c r="D305" s="2"/>
-      <c r="E305" s="2"/>
-      <c r="F305" s="2"/>
-      <c r="G305" s="2"/>
-      <c r="H305" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -6166,18 +6108,18 @@
     <mergeCell ref="C95:G95"/>
     <mergeCell ref="C108:G108"/>
     <mergeCell ref="C125:G125"/>
-    <mergeCell ref="C141:G141"/>
-    <mergeCell ref="C158:G158"/>
-    <mergeCell ref="C174:G174"/>
-    <mergeCell ref="C189:G189"/>
-    <mergeCell ref="C197:G197"/>
-    <mergeCell ref="C211:G211"/>
-    <mergeCell ref="C225:G225"/>
-    <mergeCell ref="C242:G242"/>
-    <mergeCell ref="C259:G259"/>
-    <mergeCell ref="C276:G276"/>
-    <mergeCell ref="C290:G290"/>
-    <mergeCell ref="C297:G297"/>
+    <mergeCell ref="C138:G138"/>
+    <mergeCell ref="C155:G155"/>
+    <mergeCell ref="C171:G171"/>
+    <mergeCell ref="C186:G186"/>
+    <mergeCell ref="C194:G194"/>
+    <mergeCell ref="C208:G208"/>
+    <mergeCell ref="C222:G222"/>
+    <mergeCell ref="C239:G239"/>
+    <mergeCell ref="C256:G256"/>
+    <mergeCell ref="C273:G273"/>
+    <mergeCell ref="C287:G287"/>
+    <mergeCell ref="C294:G294"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Label Module 8 as DBQ
</commit_message>
<xml_diff>
--- a/exports/US History 8-1 - Course Outline.xlsx
+++ b/exports/US History 8-1 - Course Outline.xlsx
@@ -2749,7 +2749,7 @@
       </c>
       <c r="C125" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ratification &amp; How the Constitution Works</t>
+          <t xml:space="preserve">Ratification &amp; How the Constitution Works (DBQ)</t>
         </is>
       </c>
       <c r="D125" s="16"/>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Ratification &amp; How the Constitution Works</t>
+          <t xml:space="preserve">Overview | Ratification &amp; How the Constitution Works (DBQ)</t>
         </is>
       </c>
       <c r="D126" s="5"/>

</xml_diff>